<commit_message>
update the context DB
</commit_message>
<xml_diff>
--- a/context_DB/AFG_context_db.xlsx
+++ b/context_DB/AFG_context_db.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BL35"/>
+  <dimension ref="A1:BM35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -686,65 +686,70 @@
       </c>
       <c r="AZ1" s="1" t="inlineStr">
         <is>
+          <t>fatalities</t>
+        </is>
+      </c>
+      <c r="BA1" s="1" t="inlineStr">
+        <is>
+          <t>event_count_evt2</t>
+        </is>
+      </c>
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>ADM2_PCODE_evt2</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>ADM3_PCODE_evt2</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>event_type</t>
+        </is>
+      </c>
+      <c r="BE1" s="1" t="inlineStr">
+        <is>
+          <t>sub_event_type</t>
+        </is>
+      </c>
+      <c r="BF1" s="1" t="inlineStr">
+        <is>
+          <t>actor1</t>
+        </is>
+      </c>
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
+          <t>assoc_actor_1</t>
+        </is>
+      </c>
+      <c r="BH1" s="1" t="inlineStr">
+        <is>
+          <t>actor2</t>
+        </is>
+      </c>
+      <c r="BI1" s="1" t="inlineStr">
+        <is>
+          <t>assoc_actor_2</t>
+        </is>
+      </c>
+      <c r="BJ1" s="1" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="BK1" s="1" t="inlineStr">
+        <is>
+          <t>event_date</t>
+        </is>
+      </c>
+      <c r="BL1" s="1" t="inlineStr">
+        <is>
           <t>admin2</t>
         </is>
       </c>
-      <c r="BA1" s="1" t="inlineStr">
-        <is>
-          <t>fatalities</t>
-        </is>
-      </c>
-      <c r="BB1" s="1" t="inlineStr">
-        <is>
-          <t>event_count_evt2</t>
-        </is>
-      </c>
-      <c r="BC1" s="1" t="inlineStr">
-        <is>
-          <t>ADM3_PCODE_evt2</t>
-        </is>
-      </c>
-      <c r="BD1" s="1" t="inlineStr">
-        <is>
-          <t>event_type</t>
-        </is>
-      </c>
-      <c r="BE1" s="1" t="inlineStr">
-        <is>
-          <t>sub_event_type</t>
-        </is>
-      </c>
-      <c r="BF1" s="1" t="inlineStr">
-        <is>
-          <t>actor1</t>
-        </is>
-      </c>
-      <c r="BG1" s="1" t="inlineStr">
-        <is>
-          <t>assoc_actor_1</t>
-        </is>
-      </c>
-      <c r="BH1" s="1" t="inlineStr">
-        <is>
-          <t>actor2</t>
-        </is>
-      </c>
-      <c r="BI1" s="1" t="inlineStr">
-        <is>
-          <t>assoc_actor_2</t>
-        </is>
-      </c>
-      <c r="BJ1" s="1" t="inlineStr">
-        <is>
-          <t>notes</t>
-        </is>
-      </c>
-      <c r="BK1" s="1" t="inlineStr">
-        <is>
-          <t>event_date</t>
-        </is>
-      </c>
-      <c r="BL1" s="1" t="inlineStr">
+      <c r="BM1" s="1" t="inlineStr">
         <is>
           <t>ratio IDP/ToTN - HPC2025</t>
         </is>
@@ -818,47 +823,158 @@
       <c r="W2" t="n">
         <v>34.28</v>
       </c>
-      <c r="X2" t="inlineStr"/>
-      <c r="Y2" t="inlineStr"/>
-      <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr"/>
-      <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="inlineStr"/>
-      <c r="AD2" t="inlineStr"/>
-      <c r="AE2" t="inlineStr"/>
-      <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr"/>
-      <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="inlineStr"/>
-      <c r="AK2" t="inlineStr"/>
-      <c r="AL2" t="inlineStr"/>
-      <c r="AM2" t="inlineStr"/>
-      <c r="AN2" t="inlineStr"/>
-      <c r="AO2" t="inlineStr"/>
-      <c r="AP2" t="inlineStr"/>
-      <c r="AQ2" t="inlineStr"/>
-      <c r="AR2" t="inlineStr"/>
-      <c r="AS2" t="inlineStr"/>
-      <c r="AT2" t="inlineStr"/>
-      <c r="AU2" t="inlineStr"/>
-      <c r="AV2" t="inlineStr"/>
+      <c r="X2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>4</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN2" t="n">
+        <v>5</v>
+      </c>
+      <c r="AO2" t="inlineStr">
+        <is>
+          <t>2025-02-24 ---- 2024-10-20 ---- 2024-09-02 ---- 2024-07-20 ---- 2024-01-10</t>
+        </is>
+      </c>
+      <c r="AP2" t="inlineStr">
+        <is>
+          <t>February 2025: An educator was arrested from his home by four members of the Taliban for campaigning for the education rights of girls. ---- October 2024: An educator was arrested by the Taliban.  ---- September 2024: A university professor and other people were killed and 13-59 people injured when an IS suicide bomb targeted the Taliban government‚Äôs prosecution service. The bomber waited until government employees finished their shifts and then detonated the explosive in the middle of a crowd. IS claimed the attack was revenge for ‚ÄúMuslims held in Taliban prisons‚Äù.  ---- July 2024: The head of a university faculty was detained by Taliban intelligence. Photos show the lecturer had been beaten. He was threatened with arrest by the Taliban in the past on accusations of speaking to foreign media.  ---- January 2024: Taliban forces arrested the administrative deputy head of a university, for offering online education to women and girls in Afghanistan. The university was established in December 2022 after the Taliban's ban on women's education.</t>
+        </is>
+      </c>
+      <c r="AQ2" t="inlineStr">
+        <is>
+          <t>Home ---- Unspecified Location ---- Unspecified Location ---- Unspecified Location</t>
+        </is>
+      </c>
+      <c r="AR2" t="inlineStr">
+        <is>
+          <t>Other ---- Police ---- NSA ---- Police ---- Police</t>
+        </is>
+      </c>
+      <c r="AS2" t="inlineStr">
+        <is>
+          <t>Islamic Emirate of Afghanistan ---- Islamic Emirate of Afghanistan ---- Islamic State ---- Islamic Emirate of Afghanistan ---- Islamic Emirate of Afghanistan</t>
+        </is>
+      </c>
+      <c r="AT2" t="inlineStr">
+        <is>
+          <t>Firearms ---- No Information on the Weapon Used ---- SVIED ---- Firearms ---- Firearms</t>
+        </is>
+      </c>
+      <c r="AU2" t="inlineStr">
+        <is>
+          <t>Not Applicable ---- Not Applicable ---- Not Applicable ---- Not Applicable ---- Not Applicable</t>
+        </is>
+      </c>
+      <c r="AV2" t="inlineStr">
+        <is>
+          <t>NoInformation ---- NoInformation ---- NoInformation ---- NoInformation</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr"/>
       <c r="AX2" t="inlineStr"/>
-      <c r="AY2" t="inlineStr"/>
-      <c r="AZ2" t="inlineStr"/>
-      <c r="BA2" t="inlineStr"/>
-      <c r="BB2" t="inlineStr"/>
+      <c r="AY2" t="inlineStr">
+        <is>
+          <t>Kabul</t>
+        </is>
+      </c>
+      <c r="AZ2" t="n">
+        <v>26</v>
+      </c>
+      <c r="BA2" t="n">
+        <v>40</v>
+      </c>
+      <c r="BB2" t="inlineStr">
+        <is>
+          <t>AF0101</t>
+        </is>
+      </c>
       <c r="BC2" t="inlineStr"/>
-      <c r="BD2" t="inlineStr"/>
-      <c r="BE2" t="inlineStr"/>
-      <c r="BF2" t="inlineStr"/>
-      <c r="BG2" t="inlineStr"/>
-      <c r="BH2" t="inlineStr"/>
-      <c r="BI2" t="inlineStr"/>
-      <c r="BJ2" t="inlineStr"/>
-      <c r="BK2" t="inlineStr"/>
-      <c r="BL2" t="n">
+      <c r="BD2" t="inlineStr">
+        <is>
+          <t>Strategic developments ---- Violence against civilians ---- Protests ---- Strategic developments ---- Battles ---- Strategic developments ---- Violence against civilians ---- Violence against civilians ---- Strategic developments ---- Violence against civilians ---- Battles ---- Protests ---- Violence against civilians ---- Violence against civilians ---- Violence against civilians ---- Violence against civilians ---- Violence against civilians ---- Explosions/Remote violence ---- Protests ---- Strategic developments ---- Violence against civilians ---- Protests ---- Violence against civilians ---- Violence against civilians ---- Violence against civilians ---- Violence against civilians ---- Strategic developments ---- Strategic developments ---- Violence against civilians ---- Violence against civilians ---- Strategic developments ---- Violence against civilians ---- Strategic developments ---- Strategic developments ---- Violence against civilians ---- Violence against civilians ---- Strategic developments ---- Strategic developments ---- Strategic developments ---- Strategic developments</t>
+        </is>
+      </c>
+      <c r="BE2" t="inlineStr">
+        <is>
+          <t>Other ---- Abduction/forced disappearance ---- Peaceful protest ---- Arrests ---- Armed clash ---- Looting/property destruction ---- Attack ---- Attack ---- Other ---- Attack ---- Armed clash ---- Peaceful protest ---- Abduction/forced disappearance ---- Abduction/forced disappearance ---- Abduction/forced disappearance ---- Attack ---- Attack ---- Suicide bomb ---- Peaceful protest ---- Other ---- Abduction/forced disappearance ---- Peaceful protest ---- Abduction/forced disappearance ---- Attack ---- Attack ---- Attack ---- Other ---- Other ---- Attack ---- Attack ---- Other ---- Abduction/forced disappearance ---- Other ---- Other ---- Abduction/forced disappearance ---- Attack ---- Other ---- Other ---- Other ---- Other</t>
+        </is>
+      </c>
+      <c r="BF2" t="inlineStr">
+        <is>
+          <t>Government of Afghanistan (2021-) ---- Military Forces of Afghanistan (2021-) ---- Protesters (Afghanistan) ---- Military Forces of Afghanistan (2021-) ---- National Resistance Front ---- Police Forces of Afghanistan (2021-) ---- Military Forces of Afghanistan (2021-) ---- Police Forces of Afghanistan (2021-) General Directorate of Intelligence ---- Government of Afghanistan (2021-) ---- Military Forces of Afghanistan (2021-) ---- National Resistance Front ---- Protesters (Afghanistan) ---- Military Forces of Afghanistan (2021-) ---- Police Forces of Afghanistan (2021-) General Directorate of Intelligence ---- Police Forces of Afghanistan (2021-) General Directorate of Intelligence ---- Military Forces of Afghanistan (2021-) ---- Police Forces of Afghanistan (2021-) Vice and Virtue Department ---- Islamic State Khorasan Province (ISKP) ---- Protesters (Afghanistan) ---- Government of Afghanistan (2021-) ---- Police Forces of Afghanistan (2021-) General Directorate of Intelligence ---- Protesters (Afghanistan) ---- Military Forces of Afghanistan (2021-) ---- Unidentified Armed Group (Afghanistan) ---- Police Forces of Afghanistan (2021-) Vice and Virtue Department ---- Police Forces of Afghanistan (2021-) General Directorate of Intelligence ---- Government of Afghanistan (2021-) ---- Government of Afghanistan (2021-) ---- Military Forces of Afghanistan (2021-) ---- Military Forces of Afghanistan (2021-) ---- Military Forces of Afghanistan (2021-) ---- Police Forces of Afghanistan (2021-) General Directorate of Intelligence ---- Government of Afghanistan (2021-) ---- Government of Afghanistan (2021-) ---- Police Forces of Afghanistan (2021-) General Directorate of Intelligence ---- Military Forces of Afghanistan (2021-) ---- Government of Afghanistan (2021-) ---- Government of Afghanistan (2021-) ---- Government of Afghanistan (2021-) ---- Government of Afghanistan (2021-)</t>
+        </is>
+      </c>
+      <c r="BG2" t="inlineStr">
+        <is>
+          <t>Students (Afghanistan); Women (Afghanistan) ---- Teachers (Afghanistan); Women (Afghanistan) ---- Women (Afghanistan) ---- Women (Afghanistan) ---- Military Forces of Afghanistan (2021-) ---- Police Forces of Afghanistan (2021-) General Directorate of Intelligence</t>
+        </is>
+      </c>
+      <c r="BH2" t="inlineStr">
+        <is>
+          <t>Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Military Forces of Afghanistan (2021-) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Military Forces of Afghanistan (2021-) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BI2" t="inlineStr">
+        <is>
+          <t>Women (Afghanistan) ---- Students (Afghanistan) ---- Students (Afghanistan); Women (Afghanistan) ---- Journalists (Afghanistan); Teachers (Afghanistan) ---- Militia (Alipour); Teachers (Afghanistan) ---- Government of Afghanistan (2021-); Women (Afghanistan) ---- Teachers (Afghanistan) ---- Students (Afghanistan) ---- Teachers (Afghanistan) ---- Labor Group (Afghanistan); Teachers (Afghanistan); Government of Afghanistan (2021-) ---- Teachers (Afghanistan) ---- Pashtun Ethnic Group (Afghanistan); PTM: Pashtun Protection Movement; Teachers (Afghanistan) ---- Teachers (Afghanistan) ---- Teachers (Afghanistan) ---- Students (Afghanistan) ---- Health Workers (Afghanistan); Students (Afghanistan); Women (Afghanistan) ---- Labor Group (Afghanistan); Teachers (Afghanistan); Women (Afghanistan) ---- Hazara Ethnic Group (Afghanistan); Prisoners (Afghanistan); Teachers (Afghanistan); Shiite Muslim Group (Afghanistan) ---- Hazara Ethnic Group (Afghanistan); Prisoners (Afghanistan); Shiite Muslim Group (Afghanistan); Teachers (Afghanistan) ---- Muslim Group (Afghanistan); Teachers (Afghanistan) ---- Journalists (Afghanistan); Women (Afghanistan) ---- Students (Afghanistan); Teachers (Afghanistan) ---- Teachers (Afghanistan) ---- Students (Afghanistan) ---- Women (Afghanistan); Health Workers (Afghanistan) ---- Students (Afghanistan); Women (Afghanistan) ---- Teachers (Afghanistan); Women (Afghanistan) ---- Labor Group (Afghanistan); Teachers (Afghanistan); Women (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BJ2" t="inlineStr">
+        <is>
+          <t>Other: Around 9 January 2024 (as reported), the Ministry of Promotion of Virtue and Prevention of Vice imposed an Islamic dress code in PD18 area of Kabul, after a meeting with local school principals. The new order restricted women from wearing short skirts above the knee, small head scarves, and tight or short leggings or pants. ---- On 10 January 2024, Taliban forces arrested the administrative deputy head of Roshan Afghanistan Online University in Kabul, for offering online education to women and girls in Afghanistan. The university was established in December 2022 after the Taliban's ban on women's education. His whereabouts remained unknown. ---- Around 21 January 2024 (as reported), a group of female students conducted an indoor protest in Kabul province, denouncing the restrictions of women's rights and arbitrary arrest of women on charges of wearing improper Hijab. ---- On 11 March 2024, Taliban forces arrested 15 boys and 5 girls in Dasht-e-Barchi area of Kabul city, who were suspected of being students of an education center. Motive behind their arrest remained unknown. ---- On 29 March 2024, three Taliban members were killed and three were wounded following two attacks by National Resistance Front militants in Kabul city. Two Taliban members were killed and one was wounded in the first attack on a checkpoint near the Kot-e Sangi bridge in PD5, while one was killed and one was wounded in the second attack near the Habibia High School of PD7. ---- Property destruction: On 1 April 2024, Taliban morality police closed an arts workshop and three private tuition centers in PD7 and PD10 of Kabul city because female students above the sixth grade attended classes. Taliban members destroyed paintings and artworks in the workshop. Taliban prevented girls above the sixth grade from education since their takeover of power in Afghanistan in August 2021. ---- On 24 April 2024, Taliban forces raided the home of the owner of Noorin TV, Noorin University, and a school in Kabul city, and pushed him from the third floor in an attempt to kill him. While he survived, he sustained critical injuries and was later transferred to Pakistan for medical treatment. ---- Around 21 May 2024 (week of), a teacher was arrested by Taliban intelligence forces from Qalah-ye Now area in Dasht Barchi of Kabul city, in accusation of collaborating with Alipour militia. He is a resident of Hissa-e-awali Behsud district and was tortured while being held in Taliban intelligence prison in Wardak province. ---- Other: Around 1 June 2024 (beginning of month), Taliban's Supreme Leader ordered the salary for all women employed in government positions to be set at 5,000 Afghanis per month regardless of their job, qualifications, or experience (coded to Kabul). Taliban initially barred women from being employed in public sector except for some positions that cannot be done by men, according to group's interpretation of Islamic law (nurses, teachers etc.). The decision results in at least 75 percent of drop in women's salaries. ---- On 19 June 2024, Taliban forces interrogated, beat and tortured a young man, who was a student in Iran, at a checkpoint in Kabul-Kandahar highway [coded to Kabul province], for carrying Farsi books about Ahmad Shah Masoud and poetry books, and set his books on fire. According to sources, Taliban intended to shoot him, but he was released after the mediation of an elder. ---- On 3 July 2024, two Taliban members were killed and one was wounded following an attack by National Resistance Front militants near the Zulfikar School of PD6, Kabul city. In another attack, one Taliban commander was killed and two members were wounded following an attack on their checkpoint in PD17. NRF said their militants did not suffer casualties. ---- Around 3 July 2024 (as reported), teachers, all women, held protests n Kabul city against Taliban's salary cuts for women public sector workers. ---- On 18 July 2024, a civilian, the son of the principal of Ghulam Haider Khan High School, was arrested by Taliban in PD15 of Kabul city. His whereabouts remained unknown. ---- On 21 July 2024, Taliban intelligence arrested a university professor near Ibn Sina Private University in the Red Bridge/Pulsarukh area of Kabul city. His family said he was beaten by the Taliban during arrest. His whereabouts remained unknown. He was threatened by Taliban in the past for speaking to foreign media. ---- Around 5 August 2024, Taliban intelligence forces arrested a social media activist at Hamid Karzai International Airport, Kabul, upon his return from Dubai. His whereabouts remained unknown. While the motive behind his arrest is unclear, he had supported girls' education and Afghanistan's tricolor flag on social media, despite being a Taliban supporter. ---- On 13 August 2024, one university student was shot and killed by a Taliban member in the Karta-e-Now area of Kabul city. The Taliban member was arrested. There were conflicting reports about the motive, with some sources claiming that the victim was shot at when his vehicle passed by a Taliban convoy. The Taliban claimed it was an accidental shooting and later handed over 200,000 Afghanis to the victim's father. ---- On 16 August 2024, a teacher was severely beaten by Taliban Vice and Virtue members in Kabul city, for teaching English to girls over the age of 15 at an educational center. The Taliban have prohibited girls from attending school beyond the sixth grade. ---- On 2 September 2024, IS militants conducted a suicide bomb attack targeting a specific group of employees near the former attorney general's office in the sixth security zone of Qala Bakhtiar area in Kabul-Darul Aman city (Kabul). 16-34 civilians including a veteran employee, university professor and woman were killed and 13-59 were left injured. While Taliban claimed that 6 civilians were killed and 13 were wounded, IS claimed that more than 45 including Taliban members were killed and wounded. The Afghanistan Prosecutors' Association confirmed the deaths of 16 prosecutors in the attack. Fatalities coded as 17 including the suicide bomber. ---- On 11 September 2024, more than 10 women from the Afghanistan Women's History Change Movement protested in the Dasht Barchi area of Kabul city, demanding basic rights and freedoms while opposing the international community's decision to hand over Afghan embassies to the Taliban. They held slogans such as 'Taliban commit crimes, the world supports' and 'Education, work, freedom.' ---- Other: Around 11 September 2024 (as reported), Taliban Ministry of Education announced that 21,257 religious schools were established across the country [coded to Kabul], with 3,687,200 individuals currently engaged in learning Islamic teachings. It's unclear if girls are allowed to attend these schools, although the Taliban permitted girls to attend religious schools last year. ---- On 11 September 2024, Taliban intelligence arrested deputy dean/vice president of Karwan University from the university in Kabul city. His whereabouts remained unknown. ---- On 25 September 2024, members of the Historical Transformation Movement, a women's movement, held a protest in Kabul city, to demand their rights including work and education. The protest lasted for 30 minutes out of concern for their safety. ---- On 20 October 2024, a university professor and political expert was arrested by the Taliban in Kabul province. The reason for his arrest and his whereabouts remained unknown. A few days earlier, he had claimed that the Taliban removed his name from the list of verified experts allowed to participate in media programs. An image of the professor carrying a red hat (affiliated with the Pashtun Protection Movement), was circulating on social media. His release was reported on 21 November. ---- On 30 October 2024, a private school director was killed by unknown gunmen in his office in the Familihay Rishkhor area of PD7, Kabul city. The motive remained unclear. The school operates in the building owned by the former head of the army staff. Despite multiple appeals from the victim's family, the Taliban have not taken steps to identify the perpetrators. ---- On 30 November 2024, a painting teacher was severely beaten by unknown gunmen (likely Taliban Vice and Virtue members, given his prior arrest by them for painting living beings and teaching girls) in the Tank Tel area of Dasht-e Barchi in PD13 of Kabul city. The teacher stated that he had closed his painting workshop due to the pressure from the Taliban. The Taliban's 'Vice and Virtue' law banned the publication of images of living beings. ---- On 1 December 2024, two civil society activists, one of whom was also a Kabul University student, were arrested by Taliban intelligence forces from the Dasht-e-Barchi area and the Kabul University dormitory in Kabul city. The student was also beaten by the Taliban dormitory director. The motive behind their arrest remained unknown, but both had participated in women's advocacy protests, demanding women's rights and an end to the Hazara genocide. The student was a resident of Khedir district, Daykundi. Their whereabouts remained unknown. The student was later released on 11 January 2025 on bail, while the other activist remained in custody. After his release, he returned to Kabul University, but university officials informed him that he had been expelled. He was subsequently summoned again by the Taliban, but fearing re-imprisonment, he managed to leave the country. The Taliban also seized his laptop and electronic ID card. ---- Other: On 2 December 2024, the Taliban Ministry of Public Health, under the directive of the Taliban's supreme leader ordered the closure of all public and private medical institutes for female medical education (coded to Kabul) until further notice. This order barred all institutions from enrolling or teaching female students in midwifery, dentistry, nursing, and laboratory sciences. The Taliban have already banned girls from attending school and university for more than three years. At least 35,000 female students, enrolled in 10 government institutes and over 150 private ones, have been deprived of their education due to the ban. ---- Other: Around 8 December 2024 (as reported), Taliban gave female employees in Afghan universities a three days notice to have a male relative assume their duties or stated that they would be dismisssed [coded to Kabul]. ---- Around 26 December 2024 (as reported), the Taliban beat and mistreated the families of Kabul University students while prohibiting them from attending the graduation ceremony in Kabul province, despite collecting 1,500 Afghanis from each student. The Taliban also barred students from filming the event and wearing graduation attire. ---- Around 15 January 2025 (as reported), a Hazara teacher (likely following Shia Islam based on location) was arrested in a nighttime raid in Kabul city on charges of posting critical content about the Taliban. During his detention, he was severely tortured, resulting in broken teeth and a brief hospitalization due to his deteriorating health. Later, the Taliban's primary court sentenced him to seven years in prison for running a fake Facebook account and opposing their regime. He was originally from Bamyan province. ---- Other: Around 19 January 2025 (as reported), a Shia Hazara civil rights activist and teacher died after his release due to severe torture endured while in Taliban custody in Kabul city. On 9 February 2023, he was arrested by the Taliban in the Dasht-e-Barchi area of Kabul and sentenced to three years and two months in prison. He was subjected to continuous and severe torture during his detention. He was later released on 25 July 2024, but succumbed to the effects of the torture. He was a prominent member of the Tabassum Movement-established in 2015 following the execution of seven Hazara Shiites by unknown armed groups-and the Enlightenment Movement, which opposed the former republic government's perceived anti-Hazara discrimination after the rerouting of a power line from Bamyan to Salang. He also served as a commander in the public uprisings in Mazar-e-Sharif. After the Taliban takeover, he became an active participant in protests in Kabul, advocating for human rights and women's rights while criticizing Taliban policies, which motivated his arrest. ---- On 26 January 2025, Taliban intelligence forces arrested a teacher and head of a private religious school near his home in the 315 area of Kabul city. He is a resident of Tawakh village in Unaba district, Panjshir. The motive behind his arrest and his whereabouts remained unknown. ---- Other: On 4 February 2025, the Taliban's Ministry of Information and Culture announced the suspension of Begum and Jawanan Radios, two independent media outlets owned by the same person, pending further investigation. The ministry cited multiple violations of media regulations and improper use of its license, including providing content to a foreign-based television station. Taliban intelligence and ministry employees stormed the Begum Radio office and Radio Jawanan, located in the Wazir Akbar Khan area of Kabul province, and interrogated the staff. Two male journalists, one from each station, were arrested. Taliban forces also seized computers, hard drives, documents, and mobile phones from female journalists and two male employees. Begum Radio, a women-run station focused on women's issues and dedicated to women's empowerment and education, was founded on March 8, 2021, by entrepreneur and journalist Hamida Aman. After receiving a broadcasting license from the Taliban in December 2021, it aired educational programs for students, particularly targeting girls who have been barred from formal education since the Taliban's takeover. Radio Jawanan, established in 2011, aimed to raise civic awareness and promote dialogue between people and cultures. On 22 February 2025, the Taliban announced that it had re-authorized Both Radios to resume operations, provided they adhered to the group's principles and regulations and avoided future violations. However, the Afghanistan Journalists Center (AFJC) reported that the station's offices remain closed and that the two detained journalists have not yet been released. According to reports, one of them remained in custody under the Taliban's intelligence directorate, with his condition unknown. Later, AFJC confirmed that on 16 march 2025, both radios resumed broadcasting. ---- Other: On 20 February 2025, the Taliban, under orders from their leader Hibatullah Akhundzada, mandated a uniform policy for male students and teachers in schools across all provinces (coded to Kabul). The regulation consists of nine articles and four sections and is to be implemented nationwide. According to the directive, students in grades 1 to 9 must wear blue shalwar kameez (a long tunic and trousers as traditional Afghan clothing) with a white cap, while students in grades 10 to 12 are required to wear white shalwar kameez with a turban. Teachers must also wear shalwar kameez with either a cap or turban. This policy has led to student dropouts and forced expulsions, with no exceptions made for economic hardship or personal discomfort. Traditionally, such attire was exclusive to religious school students. ---- Around 25 February 2025 (as reported), Taliban intelligence forces arrested an education activist in Kabul province. The motive for his arrest and his whereabouts remained unknown. He had been providing free schooling to girls and children in remote areas of Kabul and several other provinces. ---- On 17 April 2025, a Taliban high school headmaster whipped several students in the Shah Shahid area of Kabul city, for failing to comply with the Taliban's mandatory uniform policy. ---- Other: Around 21 April 2025 (as reported), the Taliban Ministry of Public Health issued an order to shut down 11 health institutes for providing training to women and girls in Kabul. The institutes taught female students basic medical and first-aid education. A Taliban order claimed the closure was 'due to lack of permission.' ---- Other: Around 27 April 2025 (as reported), the Taliban's Ministry for the Promotion of Virtue and Prevention of Vice warned private schools in Kabul province that female students who do not observe the Islamic hijab would be arrested and detained for two to three days. If no one guarantees their release, the authorities would formalize their cases and imprison them in Pul-e-Charkhi prison (Afghanistan's largest and most dangerous detention facility). The Taliban instructed school directors to tell female students to wear clothing that covers below the knees to avoid arrest. ---- Other: Around 12 May 2025 (as reported), the Taliban reduced the positions of female university professors (coded to Kabul). Several sources said that the move is systematic exclusion and gender apartheid in Afghanistan. This action is part of a broader directive from Taliban leader Hibatullah Akhundzada to downsize thousands of government positions amid foreign aid cuts and budget shortfalls. The Taliban's Ministry of Higher Education cut around 14 percent of its workforce, with the majority of the reductions targeting women. ---- Other: Around 20 May 2025 (as reported), the Taliban dismissed around 120 female teachers and staff from kindergartens in Kabul city. The affected employees had not received salaries for the past three months and are facing severe financial hardship. This action is part of a broader directive from Taliban leader Hibatullah Akhundzada to downsize thousands of government positions amid foreign aid cuts and budget shortfalls. The Taliban's Ministry of Higher Education cut around 14 percent of its workforce, with the majority of the reductions targeting women.</t>
+        </is>
+      </c>
+      <c r="BK2" t="inlineStr">
+        <is>
+          <t>2024-01-09 ---- 2024-01-10 ---- 2024-01-21 ---- 2024-03-11 ---- 2024-03-29 ---- 2024-04-01 ---- 2024-04-24 ---- 2024-05-21 ---- 2024-06-01 ---- 2024-06-19 ---- 2024-07-03 ---- 2024-07-03 ---- 2024-07-18 ---- 2024-07-21 ---- 2024-08-05 ---- 2024-08-13 ---- 2024-08-16 ---- 2024-09-02 ---- 2024-09-11 ---- 2024-09-11 ---- 2024-09-11 ---- 2024-09-25 ---- 2024-10-20 ---- 2024-10-30 ---- 2024-11-30 ---- 2024-12-01 ---- 2024-12-02 ---- 2024-12-08 ---- 2024-12-26 ---- 2025-01-15 ---- 2025-01-19 ---- 2025-01-26 ---- 2025-02-04 ---- 2025-02-20 ---- 2025-02-25 ---- 2025-04-17 ---- 2025-04-21 ---- 2025-04-27 ---- 2025-05-12 ---- 2025-05-20</t>
+        </is>
+      </c>
+      <c r="BL2" t="inlineStr"/>
+      <c r="BM2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -957,20 +1073,61 @@
       <c r="AV3" t="inlineStr"/>
       <c r="AW3" t="inlineStr"/>
       <c r="AX3" t="inlineStr"/>
-      <c r="AY3" t="inlineStr"/>
-      <c r="AZ3" t="inlineStr"/>
-      <c r="BA3" t="inlineStr"/>
-      <c r="BB3" t="inlineStr"/>
+      <c r="AY3" t="inlineStr">
+        <is>
+          <t>Kapisa</t>
+        </is>
+      </c>
+      <c r="AZ3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA3" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB3" t="inlineStr">
+        <is>
+          <t>AF0203</t>
+        </is>
+      </c>
       <c r="BC3" t="inlineStr"/>
-      <c r="BD3" t="inlineStr"/>
-      <c r="BE3" t="inlineStr"/>
-      <c r="BF3" t="inlineStr"/>
+      <c r="BD3" t="inlineStr">
+        <is>
+          <t>Violence against civilians</t>
+        </is>
+      </c>
+      <c r="BE3" t="inlineStr">
+        <is>
+          <t>Abduction/forced disappearance</t>
+        </is>
+      </c>
+      <c r="BF3" t="inlineStr">
+        <is>
+          <t>Police Forces of Afghanistan (2021-) General Directorate of Intelligence</t>
+        </is>
+      </c>
       <c r="BG3" t="inlineStr"/>
-      <c r="BH3" t="inlineStr"/>
-      <c r="BI3" t="inlineStr"/>
-      <c r="BJ3" t="inlineStr"/>
-      <c r="BK3" t="inlineStr"/>
-      <c r="BL3" t="n">
+      <c r="BH3" t="inlineStr">
+        <is>
+          <t>Civilians (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BI3" t="inlineStr">
+        <is>
+          <t>Students (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BJ3" t="inlineStr">
+        <is>
+          <t>On 27 July 2025, Taliban intelligence arrested two men including a student the Bolaghayn village of Koh Band district, Kapisa. It's unclear why they were arrested. Their whereabouts remained unknown.</t>
+        </is>
+      </c>
+      <c r="BK3" t="inlineStr">
+        <is>
+          <t>2025-07-27</t>
+        </is>
+      </c>
+      <c r="BL3" t="inlineStr"/>
+      <c r="BM3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1069,20 +1226,61 @@
       <c r="AV4" t="inlineStr"/>
       <c r="AW4" t="inlineStr"/>
       <c r="AX4" t="inlineStr"/>
-      <c r="AY4" t="inlineStr"/>
-      <c r="AZ4" t="inlineStr"/>
-      <c r="BA4" t="inlineStr"/>
-      <c r="BB4" t="inlineStr"/>
+      <c r="AY4" t="inlineStr">
+        <is>
+          <t>Parwan</t>
+        </is>
+      </c>
+      <c r="AZ4" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA4" t="n">
+        <v>5</v>
+      </c>
+      <c r="BB4" t="inlineStr">
+        <is>
+          <t>AF0302</t>
+        </is>
+      </c>
       <c r="BC4" t="inlineStr"/>
-      <c r="BD4" t="inlineStr"/>
-      <c r="BE4" t="inlineStr"/>
-      <c r="BF4" t="inlineStr"/>
+      <c r="BD4" t="inlineStr">
+        <is>
+          <t>Violence against civilians ---- Violence against civilians ---- Strategic developments ---- Violence against civilians ---- Violence against civilians</t>
+        </is>
+      </c>
+      <c r="BE4" t="inlineStr">
+        <is>
+          <t>Attack ---- Abduction/forced disappearance ---- Other ---- Abduction/forced disappearance ---- Attack</t>
+        </is>
+      </c>
+      <c r="BF4" t="inlineStr">
+        <is>
+          <t>Police Forces of Afghanistan (2021-) General Directorate of Intelligence ---- Military Forces of Afghanistan (2021-) ---- Government of Afghanistan (2021-) ---- Military Forces of Afghanistan (2021-) ---- Military Forces of Afghanistan (2021-)</t>
+        </is>
+      </c>
       <c r="BG4" t="inlineStr"/>
-      <c r="BH4" t="inlineStr"/>
-      <c r="BI4" t="inlineStr"/>
-      <c r="BJ4" t="inlineStr"/>
-      <c r="BK4" t="inlineStr"/>
-      <c r="BL4" t="n">
+      <c r="BH4" t="inlineStr">
+        <is>
+          <t>Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BI4" t="inlineStr">
+        <is>
+          <t>Journalists (Afghanistan); Prisoners (Afghanistan) ---- Former Military Forces of Afghanistan (2021-); Health Workers (Afghanistan); Students (Afghanistan) ---- Teachers (Afghanistan) ---- Students (Afghanistan) ---- Former Police Forces of Afghanistan (2021-); Teachers (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BJ4" t="inlineStr">
+        <is>
+          <t>On 13 June 2024, Taliban intelligence arrested and severely beat a former reporter in Bagram district, Parwan, for publishing a critical report on the Taliban's policies towards girls education and for a Facebook post about the Taliban using Kapisa schools as military bases. He was released on 15 June 2024. ---- On 5 August 2024, Taliban arrested a former soldier, a former military doctor, and a student in the Chaharbarj village of Jabulussaraj district, Parwan. Their whereabouts remained unknown. ---- Other: Around 3 November 2024 (as reported), the Taliban banned filming at the public university in Parwan (coded to Charikar) province, stating that all official meetings would be conducted without video recording. Sources reported that most professors at Parwan University oppose this order. The ban was enacted under the Taliban's new 'Vice and Virtue' law, which prohibits the publication of images of living beings. ---- On 13 November 2024, the son of a former jihadist commander, who is a student, was arrested by Taliban during a house search in the Gul Bahar area of Jabulussaraj district, Parwan. His whereabouts remained unknown. The Taliban had previously arrested the commander two years ago, torturing and killing him (coded separately). ---- On 26 December 2024, unidentified gunmen dressed in Taliban uniforms shot and killed a former Interior Ministry officer while he was returning from a relative's house in Toghbirdi village of Charikar city, Parwan. Motive unknown. Following the Taliban takeover, the victim had been working as a high school teacher in Charikar. Local residents claimed that Taliban members were involved in the incident, as no other armed individuals are present in Toghbirdi village. Sources also reported that the Taliban had been active in the village even before their takeover and frequently targeted former military members. The Taliban arrested a neighbor of the victim, whose two brothers are Taliban members, in connection with the incident.</t>
+        </is>
+      </c>
+      <c r="BK4" t="inlineStr">
+        <is>
+          <t>2024-06-13 ---- 2024-08-05 ---- 2024-11-03 ---- 2024-11-13 ---- 2024-12-26</t>
+        </is>
+      </c>
+      <c r="BL4" t="inlineStr"/>
+      <c r="BM4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1181,20 +1379,61 @@
       <c r="AV5" t="inlineStr"/>
       <c r="AW5" t="inlineStr"/>
       <c r="AX5" t="inlineStr"/>
-      <c r="AY5" t="inlineStr"/>
-      <c r="AZ5" t="inlineStr"/>
-      <c r="BA5" t="inlineStr"/>
-      <c r="BB5" t="inlineStr"/>
+      <c r="AY5" t="inlineStr">
+        <is>
+          <t>Wardak</t>
+        </is>
+      </c>
+      <c r="AZ5" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA5" t="n">
+        <v>3</v>
+      </c>
+      <c r="BB5" t="inlineStr">
+        <is>
+          <t>AF0407</t>
+        </is>
+      </c>
       <c r="BC5" t="inlineStr"/>
-      <c r="BD5" t="inlineStr"/>
-      <c r="BE5" t="inlineStr"/>
-      <c r="BF5" t="inlineStr"/>
+      <c r="BD5" t="inlineStr">
+        <is>
+          <t>Violence against civilians ---- Strategic developments ---- Strategic developments</t>
+        </is>
+      </c>
+      <c r="BE5" t="inlineStr">
+        <is>
+          <t>Attack ---- Other ---- Other</t>
+        </is>
+      </c>
+      <c r="BF5" t="inlineStr">
+        <is>
+          <t>Police Forces of Afghanistan (2021-) General Directorate of Intelligence ---- Government of Afghanistan (2021-) ---- Unidentified Armed Group (Afghanistan)</t>
+        </is>
+      </c>
       <c r="BG5" t="inlineStr"/>
-      <c r="BH5" t="inlineStr"/>
-      <c r="BI5" t="inlineStr"/>
-      <c r="BJ5" t="inlineStr"/>
-      <c r="BK5" t="inlineStr"/>
-      <c r="BL5" t="n">
+      <c r="BH5" t="inlineStr">
+        <is>
+          <t>Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BI5" t="inlineStr">
+        <is>
+          <t>Militia (Alipour) ---- Journalists (Afghanistan) ---- Students (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BJ5" t="inlineStr">
+        <is>
+          <t>Around 21 May 2024 (week of), an education activist was arrested by Taliban intelligence forces from Shahmardan area of Hissa-e-awali Behsud district, Wardak, in accusation of collaborating with Alipour militia. He was tortured while being held in prison in Wardak province. ---- Other: Around 18 November 2024, the Taliban's Higher Education Minister prohibited journalists from filming or photographing during his meeting at a university in Wardak (coded to Maidan Shahr) province. ---- Explosive remnants of war: On 8 April 2025, one child was killed and four school children were wounded when an old IED, remnants of war, exploded in the Zaykhaidah village of Chak-e-Wardak district, Wardak. It's unclear who planted the bomb.</t>
+        </is>
+      </c>
+      <c r="BK5" t="inlineStr">
+        <is>
+          <t>2024-05-21 ---- 2024-11-18 ---- 2025-04-08</t>
+        </is>
+      </c>
+      <c r="BL5" t="inlineStr"/>
+      <c r="BM5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1266,30 +1505,92 @@
       <c r="W6" t="n">
         <v>34.07</v>
       </c>
-      <c r="X6" t="inlineStr"/>
-      <c r="Y6" t="inlineStr"/>
-      <c r="Z6" t="inlineStr"/>
-      <c r="AA6" t="inlineStr"/>
-      <c r="AB6" t="inlineStr"/>
-      <c r="AC6" t="inlineStr"/>
-      <c r="AD6" t="inlineStr"/>
-      <c r="AE6" t="inlineStr"/>
-      <c r="AF6" t="inlineStr"/>
-      <c r="AG6" t="inlineStr"/>
-      <c r="AH6" t="inlineStr"/>
-      <c r="AI6" t="inlineStr"/>
-      <c r="AJ6" t="inlineStr"/>
-      <c r="AK6" t="inlineStr"/>
-      <c r="AL6" t="inlineStr"/>
-      <c r="AM6" t="inlineStr"/>
-      <c r="AN6" t="inlineStr"/>
-      <c r="AO6" t="inlineStr"/>
-      <c r="AP6" t="inlineStr"/>
-      <c r="AQ6" t="inlineStr"/>
-      <c r="AR6" t="inlineStr"/>
-      <c r="AS6" t="inlineStr"/>
-      <c r="AT6" t="inlineStr"/>
-      <c r="AU6" t="inlineStr"/>
+      <c r="X6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO6" t="inlineStr">
+        <is>
+          <t>2024-01-07</t>
+        </is>
+      </c>
+      <c r="AP6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">January 2024: A hand grenade was thrown into the house of the Taliban's district education chief by unidentified perpetrators, killing four of his daughters and injuring him, his wife, and son. Some reports indicated that the education worker escaped unharmed. </t>
+        </is>
+      </c>
+      <c r="AQ6" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="AR6" t="inlineStr">
+        <is>
+          <t>No Information</t>
+        </is>
+      </c>
+      <c r="AS6" t="inlineStr">
+        <is>
+          <t>No Information</t>
+        </is>
+      </c>
+      <c r="AT6" t="inlineStr">
+        <is>
+          <t>Hand Grenade</t>
+        </is>
+      </c>
+      <c r="AU6" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
       <c r="AV6" t="inlineStr"/>
       <c r="AW6" t="inlineStr"/>
       <c r="AX6" t="inlineStr"/>
@@ -1306,7 +1607,8 @@
       <c r="BI6" t="inlineStr"/>
       <c r="BJ6" t="inlineStr"/>
       <c r="BK6" t="inlineStr"/>
-      <c r="BL6" t="n">
+      <c r="BL6" t="inlineStr"/>
+      <c r="BM6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1378,47 +1680,158 @@
       <c r="W7" t="n">
         <v>42.32</v>
       </c>
-      <c r="X7" t="inlineStr"/>
-      <c r="Y7" t="inlineStr"/>
-      <c r="Z7" t="inlineStr"/>
-      <c r="AA7" t="inlineStr"/>
-      <c r="AB7" t="inlineStr"/>
-      <c r="AC7" t="inlineStr"/>
-      <c r="AD7" t="inlineStr"/>
-      <c r="AE7" t="inlineStr"/>
-      <c r="AF7" t="inlineStr"/>
-      <c r="AG7" t="inlineStr"/>
-      <c r="AH7" t="inlineStr"/>
-      <c r="AI7" t="inlineStr"/>
-      <c r="AJ7" t="inlineStr"/>
-      <c r="AK7" t="inlineStr"/>
-      <c r="AL7" t="inlineStr"/>
-      <c r="AM7" t="inlineStr"/>
-      <c r="AN7" t="inlineStr"/>
-      <c r="AO7" t="inlineStr"/>
-      <c r="AP7" t="inlineStr"/>
-      <c r="AQ7" t="inlineStr"/>
-      <c r="AR7" t="inlineStr"/>
-      <c r="AS7" t="inlineStr"/>
-      <c r="AT7" t="inlineStr"/>
-      <c r="AU7" t="inlineStr"/>
-      <c r="AV7" t="inlineStr"/>
+      <c r="X7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO7" t="inlineStr">
+        <is>
+          <t>2024-08-25</t>
+        </is>
+      </c>
+      <c r="AP7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">August 2024: A educator, social media activist and author was arrested and imprisoned by Taliban forces for criticising Taliban leaders and their policies on social media. Later, a forced confession video was released in which he expressed regret and promised to support them going forward. </t>
+        </is>
+      </c>
+      <c r="AQ7" t="inlineStr">
+        <is>
+          <t>Unspecified Location</t>
+        </is>
+      </c>
+      <c r="AR7" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="AS7" t="inlineStr">
+        <is>
+          <t>Islamic Emirate of Afghanistan</t>
+        </is>
+      </c>
+      <c r="AT7" t="inlineStr">
+        <is>
+          <t>No Information on the Weapon Used</t>
+        </is>
+      </c>
+      <c r="AU7" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="AV7" t="inlineStr">
+        <is>
+          <t>NoInformation</t>
+        </is>
+      </c>
       <c r="AW7" t="inlineStr"/>
       <c r="AX7" t="inlineStr"/>
-      <c r="AY7" t="inlineStr"/>
-      <c r="AZ7" t="inlineStr"/>
-      <c r="BA7" t="inlineStr"/>
-      <c r="BB7" t="inlineStr"/>
+      <c r="AY7" t="inlineStr">
+        <is>
+          <t>Nangarhar</t>
+        </is>
+      </c>
+      <c r="AZ7" t="n">
+        <v>10</v>
+      </c>
+      <c r="BA7" t="n">
+        <v>10</v>
+      </c>
+      <c r="BB7" t="inlineStr">
+        <is>
+          <t>AF0621</t>
+        </is>
+      </c>
       <c r="BC7" t="inlineStr"/>
-      <c r="BD7" t="inlineStr"/>
-      <c r="BE7" t="inlineStr"/>
-      <c r="BF7" t="inlineStr"/>
-      <c r="BG7" t="inlineStr"/>
-      <c r="BH7" t="inlineStr"/>
-      <c r="BI7" t="inlineStr"/>
-      <c r="BJ7" t="inlineStr"/>
-      <c r="BK7" t="inlineStr"/>
-      <c r="BL7" t="n">
+      <c r="BD7" t="inlineStr">
+        <is>
+          <t>Explosions/Remote violence ---- Explosions/Remote violence ---- Strategic developments ---- Strategic developments ---- Strategic developments ---- Strategic developments ---- Strategic developments ---- Strategic developments ---- Strategic developments ---- Violence against civilians</t>
+        </is>
+      </c>
+      <c r="BE7" t="inlineStr">
+        <is>
+          <t>Grenade ---- Remote explosive/landmine/IED ---- Arrests ---- Other ---- Other ---- Other ---- Other ---- Other ---- Other ---- Attack</t>
+        </is>
+      </c>
+      <c r="BF7" t="inlineStr">
+        <is>
+          <t>Unidentified Armed Group (Afghanistan) ---- Islamic State Khorasan Province (ISKP) ---- Military Forces of Afghanistan (2021-) ---- Military Forces of Afghanistan (2021-) ---- Government of Afghanistan (2021-) ---- Military Forces of Afghanistan (2021-) ---- Government of Afghanistan (2021-) ---- Government of Afghanistan (2021-) ---- Government of Afghanistan (2021-) ---- Unidentified Armed Group (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BG7" t="inlineStr">
+        <is>
+          <t>Police Forces of Afghanistan (2021-) General Directorate of Intelligence</t>
+        </is>
+      </c>
+      <c r="BH7" t="inlineStr">
+        <is>
+          <t>Civilians (Afghanistan) ---- Police Forces of Afghanistan (2021-) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- TTP: Tehreek-i-Taliban Pakistan ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BI7" t="inlineStr">
+        <is>
+          <t>Government of Afghanistan (2021-) ---- Civilians (Afghanistan) ---- Teachers (Afghanistan) ---- Students (Afghanistan) ---- Journalists (Afghanistan) ---- TTP-HGB: Tehreek-i-Taliban Pakistan-Hafiz Gul Bahadur ---- Students (Afghanistan); Women (Afghanistan) ---- Students (Afghanistan) ---- Students (Afghanistan); Teachers (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BJ7" t="inlineStr">
+        <is>
+          <t>On 7 January 2024, unknown armed assailants threw an hand grenade into the house of the Taliban's district education chief (mentioned as officer) in Mya Sahib village of Hesarak district, Nangarhar, leaving four of his daughters killed while his wife, son and the head of education sustained injuries. Some reports indicated that the head of education escaped unharmed. The motive remained unknown. ---- On 22 August 2024, a landmine explosion targeted the vehicle of the Taliban police commander of Nuristan in Kandak village, Darah-e-Noor District, Nangarhar, resulting in the killing of 6 civilians, including a teacher and five children from a religious school and wounding of 4 Taliban members. At least 4 family members of the Taliban police commander, including his two sons were among the killed. Some sources claimed that the commander was not in the vehicle, while others claimed he was slightly injured. Taliban officials claimed the explosion was caused by an old war remnant mine, but IS claimed responsibility for the attack, claiming they killed 4 and wounded 4 Taliban members. ---- On 25 August 2024, Taliban forces arrested and imprisoned a social media activist, author, and teacher in Shinwar district, Nangarhar, for criticizing Taliban leaders and their policies on social media. Later, a forced confession video was released in which he expressed regret for his past statements, promised not to engage in negative propaganda against the Taliban, and to support them going forward. ---- Other: On 3 November 2024, the Taliban expelled at least 50 male students from Nangarhar University in Jalalabad city, Nangarhar, for violating Taliban strict dress regulations by not wearing hats. The Taliban also warned the remaining students that they would face punishment if they failed to comply with the dress rules. ---- Other: Around 5 November 2024 (as reported), the Taliban's Higher Education Minister prohibited journalists from photographing or filming and collected students' mobile phones during a meeting at a university in Nangarhar (coded to Jalalabad) province. This restriction was enforced under the Taliban's new 'Vice and Virtue' law, which bans the publication of images of living beings. ---- Other: Around 2 December 2024 (between 25 November - 9 December), the Taliban, in coordination with their intelligence forces, began relocating TTP fighters and their families from the Pakistan-Afghanistan border areas in Shinwar, Kot, Bati Kot, Muhmand Dara, Lalpoor, and Goshta districts of Nangarhar province (coded to Jalalabad), to designated camps in Ghazni, Kabul, and northern provinces. These individuals, residing in border areas since 2015, include families associated with the Hafiz Gul Bahadur group. The phased nighttime relocations followed the killing of several TTP commanders and members in Kunar province (coded separately). Sources reported that this initiative aimed to address Pakistan's concerns over cross-border infiltration and that the Taliban in Ghazni were constructing a base for al-Qaeda and three TTP settlements with large religious schools and well-equipped dormitories. ---- Other: On 24 December 2024, the Taliban banned girls above sixth grade from attending private educational centers in Nangarhar (coded to Jalalabad) province. The provincial education department has warned that failure to comply with this order will result in serious consequences. ---- Other: Around 24 December 2024 (as reported), the Taliban, following an order from their leader Mullah Hibatullah Akhundzada, banned photography and filming at graduation ceremonies of religious schools in Nangarhar (coded to Jalalabad) province. This restriction was enforced under the Taliban's new 'Vice and Virtue' law, which prohibits the publication of images of living beings. ---- Other: On 20 April 2025, the head of the Education Faculty in Nangarhar province (coded to Jalalabad) forced students to participate in a fundraising campaign for Muslims in Gaza, requiring each student to donate 500 Afghanis. Students expressed concern over their difficult economic conditions and criticized the event, stating that organizing a pro-Palestine meeting during class hours and collecting donations by coercion is an unlawful act. ---- On 4 August 2025, 66 male students from a religious school were poisoned and hospitalized in the Channel 29 area of Muhmand Dara district, Nangarhar, after eating contaminated food with poison. Two male teachers also showed symptoms of poisoning. The reason and the perpetrators of the incident remained unknown.</t>
+        </is>
+      </c>
+      <c r="BK7" t="inlineStr">
+        <is>
+          <t>2024-01-07 ---- 2024-08-22 ---- 2024-08-25 ---- 2024-11-03 ---- 2024-11-05 ---- 2024-12-02 ---- 2024-12-24 ---- 2024-12-24 ---- 2025-04-20 ---- 2025-08-04</t>
+        </is>
+      </c>
+      <c r="BL7" t="inlineStr"/>
+      <c r="BM7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1517,20 +1930,57 @@
       <c r="AV8" t="inlineStr"/>
       <c r="AW8" t="inlineStr"/>
       <c r="AX8" t="inlineStr"/>
-      <c r="AY8" t="inlineStr"/>
-      <c r="AZ8" t="inlineStr"/>
-      <c r="BA8" t="inlineStr"/>
-      <c r="BB8" t="inlineStr"/>
+      <c r="AY8" t="inlineStr">
+        <is>
+          <t>Laghman</t>
+        </is>
+      </c>
+      <c r="AZ8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA8" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB8" t="inlineStr">
+        <is>
+          <t>AF0701</t>
+        </is>
+      </c>
       <c r="BC8" t="inlineStr"/>
-      <c r="BD8" t="inlineStr"/>
-      <c r="BE8" t="inlineStr"/>
-      <c r="BF8" t="inlineStr"/>
+      <c r="BD8" t="inlineStr">
+        <is>
+          <t>Strategic developments</t>
+        </is>
+      </c>
+      <c r="BE8" t="inlineStr">
+        <is>
+          <t>Arrests</t>
+        </is>
+      </c>
+      <c r="BF8" t="inlineStr">
+        <is>
+          <t>Police Forces of Afghanistan (2021-) General Directorate of Intelligence</t>
+        </is>
+      </c>
       <c r="BG8" t="inlineStr"/>
-      <c r="BH8" t="inlineStr"/>
+      <c r="BH8" t="inlineStr">
+        <is>
+          <t>Civilians (Afghanistan)</t>
+        </is>
+      </c>
       <c r="BI8" t="inlineStr"/>
-      <c r="BJ8" t="inlineStr"/>
-      <c r="BK8" t="inlineStr"/>
-      <c r="BL8" t="n">
+      <c r="BJ8" t="inlineStr">
+        <is>
+          <t>Around 17 July 2024, Taliban intelligence forces arrested a social media activist and comedian in Laghman [coded to Mehterlam] province for advocating the reopening of girls' schools and using satire to criticize Taliban leaders and their policies on social media. He was imprisoned, and on 17 August, a forced confession video was released, where he expressed remorse and pleaded for forgiveness. He is still being held by the Taliban.</t>
+        </is>
+      </c>
+      <c r="BK8" t="inlineStr">
+        <is>
+          <t>2024-07-17</t>
+        </is>
+      </c>
+      <c r="BL8" t="inlineStr"/>
+      <c r="BM8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1602,47 +2052,154 @@
       <c r="W9" t="n">
         <v>36.56</v>
       </c>
-      <c r="X9" t="inlineStr"/>
-      <c r="Y9" t="inlineStr"/>
-      <c r="Z9" t="inlineStr"/>
-      <c r="AA9" t="inlineStr"/>
-      <c r="AB9" t="inlineStr"/>
-      <c r="AC9" t="inlineStr"/>
-      <c r="AD9" t="inlineStr"/>
-      <c r="AE9" t="inlineStr"/>
-      <c r="AF9" t="inlineStr"/>
-      <c r="AG9" t="inlineStr"/>
-      <c r="AH9" t="inlineStr"/>
-      <c r="AI9" t="inlineStr"/>
-      <c r="AJ9" t="inlineStr"/>
-      <c r="AK9" t="inlineStr"/>
-      <c r="AL9" t="inlineStr"/>
-      <c r="AM9" t="inlineStr"/>
-      <c r="AN9" t="inlineStr"/>
-      <c r="AO9" t="inlineStr"/>
-      <c r="AP9" t="inlineStr"/>
-      <c r="AQ9" t="inlineStr"/>
-      <c r="AR9" t="inlineStr"/>
-      <c r="AS9" t="inlineStr"/>
-      <c r="AT9" t="inlineStr"/>
-      <c r="AU9" t="inlineStr"/>
-      <c r="AV9" t="inlineStr"/>
+      <c r="X9" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG9" t="n">
+        <v>3</v>
+      </c>
+      <c r="AH9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN9" t="n">
+        <v>4</v>
+      </c>
+      <c r="AO9" t="inlineStr">
+        <is>
+          <t>2025-02-27 ---- 2024-10-07 ---- 2024-09-29 ---- 2024-05-04</t>
+        </is>
+      </c>
+      <c r="AP9" t="inlineStr">
+        <is>
+          <t>February 2025: A teacher from was detained by Taliban officials. ---- October 2024: An educator was arrested by the Taliban during house search operations following a recent attack on a Taliban military base. ---- September 2024: A school was set on fire by three people, two of which were Taliban members who claimed responsibility for the attack. ---- May 2024: A educator was arrested from their classroom by Taliban forces.</t>
+        </is>
+      </c>
+      <c r="AQ9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unspecified Location ---- Unspecified Location ---- Education Building  ---- Education Building </t>
+        </is>
+      </c>
+      <c r="AR9" t="inlineStr">
+        <is>
+          <t>Other ---- Police ---- Other ---- Police</t>
+        </is>
+      </c>
+      <c r="AS9" t="inlineStr">
+        <is>
+          <t>Islamic Emirate of Afghanistan ---- Islamic Emirate of Afghanistan ---- Islamic Emirate of Afghanistan ---- Islamic Emirate of Afghanistan</t>
+        </is>
+      </c>
+      <c r="AT9" t="inlineStr">
+        <is>
+          <t>Firearms ---- No Information on the Weapon Used ---- Arson ---- Firearms</t>
+        </is>
+      </c>
+      <c r="AU9" t="inlineStr">
+        <is>
+          <t>Not Applicable ---- Not Applicable ---- School: No Further Details ---- School: No Further Details</t>
+        </is>
+      </c>
+      <c r="AV9" t="inlineStr">
+        <is>
+          <t>NoInformation ---- NoInformation ---- NoInformation</t>
+        </is>
+      </c>
       <c r="AW9" t="inlineStr"/>
       <c r="AX9" t="inlineStr"/>
-      <c r="AY9" t="inlineStr"/>
-      <c r="AZ9" t="inlineStr"/>
-      <c r="BA9" t="inlineStr"/>
-      <c r="BB9" t="inlineStr"/>
+      <c r="AY9" t="inlineStr">
+        <is>
+          <t>Panjshir</t>
+        </is>
+      </c>
+      <c r="AZ9" t="n">
+        <v>9</v>
+      </c>
+      <c r="BA9" t="n">
+        <v>9</v>
+      </c>
+      <c r="BB9" t="inlineStr">
+        <is>
+          <t>AF0801</t>
+        </is>
+      </c>
       <c r="BC9" t="inlineStr"/>
-      <c r="BD9" t="inlineStr"/>
-      <c r="BE9" t="inlineStr"/>
-      <c r="BF9" t="inlineStr"/>
+      <c r="BD9" t="inlineStr">
+        <is>
+          <t>Violence against civilians ---- Battles ---- Violence against civilians ---- Violence against civilians ---- Violence against civilians ---- Violence against civilians ---- Violence against civilians ---- Strategic developments ---- Strategic developments</t>
+        </is>
+      </c>
+      <c r="BE9" t="inlineStr">
+        <is>
+          <t>Abduction/forced disappearance ---- Armed clash ---- Abduction/forced disappearance ---- Abduction/forced disappearance ---- Abduction/forced disappearance ---- Abduction/forced disappearance ---- Abduction/forced disappearance ---- Other ---- Arrests</t>
+        </is>
+      </c>
+      <c r="BF9" t="inlineStr">
+        <is>
+          <t>Military Forces of Afghanistan (2021-) ---- National Resistance Front ---- Military Forces of Afghanistan (2021-) ---- Police Forces of Afghanistan (2021-) General Directorate of Intelligence ---- Police Forces of Afghanistan (2021-) General Directorate of Intelligence ---- Military Forces of Afghanistan (2021-) ---- Police Forces of Afghanistan (2021-) General Directorate of Intelligence ---- Government of Afghanistan (2021-) ---- Police Forces of Afghanistan (2021-) Vice and Virtue Department</t>
+        </is>
+      </c>
       <c r="BG9" t="inlineStr"/>
-      <c r="BH9" t="inlineStr"/>
-      <c r="BI9" t="inlineStr"/>
-      <c r="BJ9" t="inlineStr"/>
-      <c r="BK9" t="inlineStr"/>
-      <c r="BL9" t="n">
+      <c r="BH9" t="inlineStr">
+        <is>
+          <t>Civilians (Afghanistan) ---- Military Forces of Afghanistan (2021-) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BI9" t="inlineStr">
+        <is>
+          <t>Teachers (Afghanistan) ---- Teachers (Afghanistan) ---- Students (Afghanistan); Teachers (Afghanistan) ---- Teachers (Afghanistan) ---- Teachers (Afghanistan) ---- Journalists (Afghanistan); Teachers (Afghanistan) ---- Students (Afghanistan); Teachers (Afghanistan) ---- Labor Group (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BJ9" t="inlineStr">
+        <is>
+          <t>On 4 May 2024, Taliban forces arrested a teacher in Frobel area of Bazarak city, Panjshir, from his classroom. The reason for his arrest and his whereabouts remained unknown. He was arrested by the Taliban for some time before this. ---- On 4 October 2024, armed clashes broke out between NRF fighters and Taliban forces after NRF carried out a mine explosion in a military squadron in the Mohammad Big Khil village in Abdullah Khel Valley of Darah district, Panjshir, resulting in the killing of at least 9 Taliban members and wounding of 11 others. National Resistance Front claimed the attack and said 13 Taliban members of the Third Battalion of the Fourth Brigade, a special unit of the Ministry of Defense, were killed and two were wounded. Taliban claimed it was caused due to a gas balloon accident at a guesthouse, claiming 6 injuries. Meanwhile, the Taliban governor's office claimed that the gunfire was due to weapon testing by their forces. Following the incident, the Taliban conducted house-to-house search operations, arresting at least 10-15 local residents. On 7 October, they arrested an additional 5-6 locals, including a former military member, a teacher, and a tribal elder. Local sources claimed that none of the detainees had any connections to armed groups. Fatalities coded as 9. ---- On 7 October 2024, a school principal was arrested by the Taliban in Abdullah Khel Valley of Darah district, Panjshir, during house-to-house search operations that followed a recent NRF attack on a Taliban military base in the district (coded separately). His whereabouts remained unknown. ---- On 17 November 2024, a school teacher and poet, a village leader, and a student were arrested by Taliban intelligence forces in the Abdullah Khel Valley of Darah district, Panjshir. The motive for their arrests and their current whereabouts remained unknown. ---- On 18 November 2024, a school teacher was arrested by Taliban intelligence forces in Mohammed Beikkhel village of Darah district, Panjshir. The motive for his arrest and his current whereabouts remained unknown. ---- On 16 January 2025, Taliban arrested a teacher in the Mohammad Baikhel village of Darah district, Panjshir. He was detained last November by Taliban intelligence and then released. His whereabouts remained unknown. ---- On 25 February 2025, a teacher and YouTuber was arrested by Taliban intelligence forces in the Faraj area of Unaba district, Panjshir, due to his activities on YouTube. He hosted cultural programs in Panjshir through his channel. He is a teacher at Rukha High School and has a background in civic activism, having also worked for a local media outlet in Panjshir. His whereabouts remained unknown. ---- Other: Around 18 May 2025 (as reported), the Taliban shut down 200 local education classes supported by UNICEF in Panjshir province (coded to Bazarak). This action has deprived 5,000 students, both boys and girls, of education and left more than 200 teachers unemployed. Taliban had already barred girls above the sixth grade from attending school and closed universities to female students. ---- On 3 August 2025, 19 employees of the Panjshir Provincial Education Department were arrested by the Taliban's Vice and Virtue forces in Panjshir province (coded to Bazarak) for having short beards. Some of the detainees have since been released on bail. The Taliban banned shaved or short beards as symbols of Western culture.</t>
+        </is>
+      </c>
+      <c r="BK9" t="inlineStr">
+        <is>
+          <t>2024-05-04 ---- 2024-10-04 ---- 2024-10-07 ---- 2024-11-17 ---- 2024-11-18 ---- 2025-01-16 ---- 2025-02-25 ---- 2025-05-18 ---- 2025-08-03</t>
+        </is>
+      </c>
+      <c r="BL9" t="inlineStr"/>
+      <c r="BM9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1714,47 +2271,154 @@
       <c r="W10" t="n">
         <v>33.31</v>
       </c>
-      <c r="X10" t="inlineStr"/>
-      <c r="Y10" t="inlineStr"/>
-      <c r="Z10" t="inlineStr"/>
-      <c r="AA10" t="inlineStr"/>
-      <c r="AB10" t="inlineStr"/>
-      <c r="AC10" t="inlineStr"/>
-      <c r="AD10" t="inlineStr"/>
-      <c r="AE10" t="inlineStr"/>
-      <c r="AF10" t="inlineStr"/>
-      <c r="AG10" t="inlineStr"/>
-      <c r="AH10" t="inlineStr"/>
-      <c r="AI10" t="inlineStr"/>
-      <c r="AJ10" t="inlineStr"/>
-      <c r="AK10" t="inlineStr"/>
-      <c r="AL10" t="inlineStr"/>
-      <c r="AM10" t="inlineStr"/>
-      <c r="AN10" t="inlineStr"/>
-      <c r="AO10" t="inlineStr"/>
-      <c r="AP10" t="inlineStr"/>
-      <c r="AQ10" t="inlineStr"/>
-      <c r="AR10" t="inlineStr"/>
-      <c r="AS10" t="inlineStr"/>
-      <c r="AT10" t="inlineStr"/>
-      <c r="AU10" t="inlineStr"/>
+      <c r="X10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL10" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN10" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO10" t="inlineStr">
+        <is>
+          <t>2024-01-16</t>
+        </is>
+      </c>
+      <c r="AP10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">January 2024: Taliban arrested two girls on charges of violating the Taliban dress code, and also wearing white boots and socks near a school. At least one remains in custody. </t>
+        </is>
+      </c>
+      <c r="AQ10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Education Building </t>
+        </is>
+      </c>
+      <c r="AR10" t="inlineStr">
+        <is>
+          <t>Police</t>
+        </is>
+      </c>
+      <c r="AS10" t="inlineStr">
+        <is>
+          <t>Islamic Emirate of Afghanistan</t>
+        </is>
+      </c>
+      <c r="AT10" t="inlineStr">
+        <is>
+          <t>Firearms</t>
+        </is>
+      </c>
+      <c r="AU10" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
       <c r="AV10" t="inlineStr"/>
-      <c r="AW10" t="inlineStr"/>
+      <c r="AW10" t="inlineStr">
+        <is>
+          <t>Freed, StillInCaptivity</t>
+        </is>
+      </c>
       <c r="AX10" t="inlineStr"/>
-      <c r="AY10" t="inlineStr"/>
-      <c r="AZ10" t="inlineStr"/>
-      <c r="BA10" t="inlineStr"/>
-      <c r="BB10" t="inlineStr"/>
+      <c r="AY10" t="inlineStr">
+        <is>
+          <t>Baghlan</t>
+        </is>
+      </c>
+      <c r="AZ10" t="n">
+        <v>3</v>
+      </c>
+      <c r="BA10" t="n">
+        <v>3</v>
+      </c>
+      <c r="BB10" t="inlineStr">
+        <is>
+          <t>AF0901</t>
+        </is>
+      </c>
       <c r="BC10" t="inlineStr"/>
-      <c r="BD10" t="inlineStr"/>
-      <c r="BE10" t="inlineStr"/>
-      <c r="BF10" t="inlineStr"/>
+      <c r="BD10" t="inlineStr">
+        <is>
+          <t>Violence against civilians ---- Battles ---- Violence against civilians</t>
+        </is>
+      </c>
+      <c r="BE10" t="inlineStr">
+        <is>
+          <t>Abduction/forced disappearance ---- Armed clash ---- Attack</t>
+        </is>
+      </c>
+      <c r="BF10" t="inlineStr">
+        <is>
+          <t>Military Forces of Afghanistan (2021-) ---- Afghanistan Freedom Front ---- Islamic State Khorasan Province (ISKP)</t>
+        </is>
+      </c>
       <c r="BG10" t="inlineStr"/>
-      <c r="BH10" t="inlineStr"/>
-      <c r="BI10" t="inlineStr"/>
-      <c r="BJ10" t="inlineStr"/>
-      <c r="BK10" t="inlineStr"/>
-      <c r="BL10" t="n">
+      <c r="BH10" t="inlineStr">
+        <is>
+          <t>Civilians (Afghanistan) ---- Police Forces of Afghanistan (2021-) General Directorate of Intelligence ---- Civilians (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BI10" t="inlineStr">
+        <is>
+          <t>Women (Afghanistan) ---- Military Forces of Afghanistan (2021-); Muslim Group (Afghanistan); Teachers (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BJ10" t="inlineStr">
+        <is>
+          <t>Around 16 January 2024 (as reported), Taliban arrested two girls on charges of violating the Taliban dress code, and also wearing white boots and socks near Mustafa Kamal School in Pul-i-Khumri city, Baghlan. While on of these girls reported to be still in the Taliban custody, the whereabout of the other girl remained unknown. No information about the identities of the girls. ---- On 30 June 2024, 2 Taliban Intelligence members were killed and 3 others were severely wounded following an attack by Afghanistan Freedom Front militants on a Taliban Intelligence education centre in Karkar mine area on the outskirts of Pul-i-Khumri city, Baghlan. AFF claimed that this centre was used to train cross-border armed groups, including Uyghurs from China and Central Asia. ---- On 7 January 2025, IS militants killed a mosque imam and religious school teacher and wounded another imam in an attack in Khawaj Khan village of Baghlan-e-Jadeed (Baghlan-e-Markazi) district, Baghlan. The victims were targeted after leaving a mosque. The injured imam, a strong supporter of the Taliban who advocated for the group in his sermons, was reported to be in critical condition.</t>
+        </is>
+      </c>
+      <c r="BK10" t="inlineStr">
+        <is>
+          <t>2024-01-16 ---- 2024-06-30 ---- 2025-01-07</t>
+        </is>
+      </c>
+      <c r="BL10" t="inlineStr"/>
+      <c r="BM10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1853,20 +2517,61 @@
       <c r="AV11" t="inlineStr"/>
       <c r="AW11" t="inlineStr"/>
       <c r="AX11" t="inlineStr"/>
-      <c r="AY11" t="inlineStr"/>
-      <c r="AZ11" t="inlineStr"/>
-      <c r="BA11" t="inlineStr"/>
-      <c r="BB11" t="inlineStr"/>
+      <c r="AY11" t="inlineStr">
+        <is>
+          <t>Bamyan</t>
+        </is>
+      </c>
+      <c r="AZ11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA11" t="n">
+        <v>5</v>
+      </c>
+      <c r="BB11" t="inlineStr">
+        <is>
+          <t>AF1001</t>
+        </is>
+      </c>
       <c r="BC11" t="inlineStr"/>
-      <c r="BD11" t="inlineStr"/>
-      <c r="BE11" t="inlineStr"/>
-      <c r="BF11" t="inlineStr"/>
+      <c r="BD11" t="inlineStr">
+        <is>
+          <t>Strategic developments ---- Violence against civilians ---- Violence against civilians ---- Strategic developments ---- Strategic developments</t>
+        </is>
+      </c>
+      <c r="BE11" t="inlineStr">
+        <is>
+          <t>Arrests ---- Attack ---- Attack ---- Arrests ---- Other</t>
+        </is>
+      </c>
+      <c r="BF11" t="inlineStr">
+        <is>
+          <t>Military Forces of Afghanistan (2021-) ---- Unidentified Armed Group (Afghanistan) ---- Military Forces of Afghanistan (2021-) ---- Military Forces of Afghanistan (2021-) ---- Government of Afghanistan (2021-)</t>
+        </is>
+      </c>
       <c r="BG11" t="inlineStr"/>
-      <c r="BH11" t="inlineStr"/>
-      <c r="BI11" t="inlineStr"/>
-      <c r="BJ11" t="inlineStr"/>
-      <c r="BK11" t="inlineStr"/>
-      <c r="BL11" t="n">
+      <c r="BH11" t="inlineStr">
+        <is>
+          <t>Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BI11" t="inlineStr">
+        <is>
+          <t>Students (Afghanistan) ---- Students (Afghanistan); Women (Afghanistan); Shiite Muslim Group (Afghanistan) ---- Civilians (United Kingdom); Prisoners (Afghanistan) ---- Civilians (United Kingdom); Civilians (United States); Labor Group (Afghanistan); Prisoners (Afghanistan); Civilians (China) ---- Hazara Ethnic Group (Afghanistan); Teachers (Afghanistan); Shiite Muslim Group (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BJ11" t="inlineStr">
+        <is>
+          <t>On 16 January 2024, Taliban forces arrested 20 boys and girls, who were studying at a private education center, from the roads near the educational center in Bamyan city. Taliban claimed that the arrests were made for violating strict hijab regulations and wearing western style clothing. No more details on the incident. ---- On 21 May 2024, at least 37 female students, ages between 12 and 22 years old, were poisoned at a religious school in the Sar-e Qol area of Yakawlang district, Bamyan. The students were transferred to a hospital, but a cause couldn't be determined. Taliban intelligence interrogated the employees of the Shiite cleric office who funds the school and prevented the families from speaking with each other at the hospital. Four students were discharged, but got worse a day later. Three locals were arrested by the Taliban. The religious school is funded and managed by the office of Ayatullah Sistani, a senior Shia scholar in Iraq. ---- On 1 February 2025, the Taliban arrested three foreign citizens, including an elderly British couple born in Sri Lanka and Singapore who also held Afghan citizenship, along with their Afghan translator and driver and a Chinese-American woman (coded separately), in the Zarin area of Yakawlang district, Bamyan. The Taliban also seized and sealed their vehicles. Taliban transferred the British couple to a maximum-security prison, where they were separated. The male detainee was beaten and chained by Taliban in prison. The British couple had returned to Afghanistan after many years and had been living in Yakawlang district for the past three years. The couple ran an organization called 'Rebuild' in Afghanistan, which provides education, training and vocational learning for children and mothers in Kabul and Bamyan for 18 years. Their children have written a letter urging the Taliban to release their parents, raising concerns over their father's worsening health, adding that he is suffering from severe chest and eye infections, as well as digestive issues, due to inadequate prison conditions. The exact motive for their arrest remained unknown, but some sources reported it was due to their travel by plane without informing the Taliban police, and that their translator had pledged to inform the Taliban of their future travels to coordinate security measures. The Taliban confirmed their arrest, stating that the couple's arrest was due to a misunderstanding over fake Afghan passports and other reasons, adding that they would be released soon following investigation. ---- On 1 February 2025, the Taliban arrested three foreign citizens, including a Chinese-American woman and an elderly British couple born in Sri Lanka and Singapore who also held Afghan citizenship, along with their Afghan translator and driver, in the Zarin area of Yakawlang district, Bamyan. Taliban transferred the British couple to a maximum-security prison, where they were separated. The male detainee was beaten and chained by Taliban in prison (coded separately). The British couple had returned to Afghanistan after many years and had been living in Yakawlang district for the past three years, while the Chinese-American citizen was their guest. The couple ran an organization called 'Rebuild' in Afghanistan, which provides education, training and vocational learning for children and mothers in Kabul and Bamyan for 18 years. The exact motive for their arrest remained unknown, but some sources reported it was due to their travel by plane without informing the Taliban police, and that their translator had pledged to inform the Taliban of their future travels to coordinate security measures. The Chinese-American woman was accused of using a drone without authorization. The Taliban confirmed their arrest, stating that the couple's arrest was due to a misunderstanding over fake Afghan passports and other reasons, adding that they would be released soon following investigation. The Chinese-American woman was released on 29 March, while the British couple remained in prison. ---- Other: Around 13 May 2025 (as reported), the Taliban eliminated 53 positions at Bamyan University in Bamyan city, including 34 cadre positions. Most of the eliminated posts were held by Hazara professors (likely following Shia Islam based on location) with master's and doctoral degrees. Some sources claimed that positions held by Pashtun professors were retained. The move is part of a broader directive issued by Taliban leader, Hibatullah Akhundzada, to downsize thousands of positions across government institutions amid foreign aid cuts and budget shortfalls.</t>
+        </is>
+      </c>
+      <c r="BK11" t="inlineStr">
+        <is>
+          <t>2024-01-16 ---- 2024-05-21 ---- 2025-02-01 ---- 2025-02-01 ---- 2025-05-13</t>
+        </is>
+      </c>
+      <c r="BL11" t="inlineStr"/>
+      <c r="BM11" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1965,20 +2670,61 @@
       <c r="AV12" t="inlineStr"/>
       <c r="AW12" t="inlineStr"/>
       <c r="AX12" t="inlineStr"/>
-      <c r="AY12" t="inlineStr"/>
-      <c r="AZ12" t="inlineStr"/>
-      <c r="BA12" t="inlineStr"/>
-      <c r="BB12" t="inlineStr"/>
+      <c r="AY12" t="inlineStr">
+        <is>
+          <t>Ghazni</t>
+        </is>
+      </c>
+      <c r="AZ12" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA12" t="n">
+        <v>2</v>
+      </c>
+      <c r="BB12" t="inlineStr">
+        <is>
+          <t>AF1101</t>
+        </is>
+      </c>
       <c r="BC12" t="inlineStr"/>
-      <c r="BD12" t="inlineStr"/>
-      <c r="BE12" t="inlineStr"/>
-      <c r="BF12" t="inlineStr"/>
+      <c r="BD12" t="inlineStr">
+        <is>
+          <t>Strategic developments ---- Violence against civilians</t>
+        </is>
+      </c>
+      <c r="BE12" t="inlineStr">
+        <is>
+          <t>Other ---- Attack</t>
+        </is>
+      </c>
+      <c r="BF12" t="inlineStr">
+        <is>
+          <t>Government of Afghanistan (2021-) ---- Kuchi Tribal Militia (Afghanistan)</t>
+        </is>
+      </c>
       <c r="BG12" t="inlineStr"/>
-      <c r="BH12" t="inlineStr"/>
-      <c r="BI12" t="inlineStr"/>
-      <c r="BJ12" t="inlineStr"/>
-      <c r="BK12" t="inlineStr"/>
-      <c r="BL12" t="n">
+      <c r="BH12" t="inlineStr">
+        <is>
+          <t>Civilians (Afghanistan) ---- Civilians (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BI12" t="inlineStr">
+        <is>
+          <t>Teachers (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BJ12" t="inlineStr">
+        <is>
+          <t>Other: Around 27 October 2024 (week of), The Taliban banned filming at the public university in Ghazni province, implementing this restriction under their new 'Vice and Virtue' law, which prohibits the publication of images of living beings. ---- Around 13 May 2025 (as reported), a group of Kuchi militia assaulted and beat residents of Wasi Mohammad village in Nawur district, Ghazni, using sticks and stones. Locals claimed that the Kuchis released their livestock onto local farmlands and had set up tents near the village school, leading to harassment of both villagers and students. The Taliban are suspected to side with the Kuchis.</t>
+        </is>
+      </c>
+      <c r="BK12" t="inlineStr">
+        <is>
+          <t>2024-10-27 ---- 2025-05-13</t>
+        </is>
+      </c>
+      <c r="BL12" t="inlineStr"/>
+      <c r="BM12" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2077,20 +2823,61 @@
       <c r="AV13" t="inlineStr"/>
       <c r="AW13" t="inlineStr"/>
       <c r="AX13" t="inlineStr"/>
-      <c r="AY13" t="inlineStr"/>
-      <c r="AZ13" t="inlineStr"/>
-      <c r="BA13" t="inlineStr"/>
-      <c r="BB13" t="inlineStr"/>
+      <c r="AY13" t="inlineStr">
+        <is>
+          <t>Paktika</t>
+        </is>
+      </c>
+      <c r="AZ13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA13" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB13" t="inlineStr">
+        <is>
+          <t>AF1201</t>
+        </is>
+      </c>
       <c r="BC13" t="inlineStr"/>
-      <c r="BD13" t="inlineStr"/>
-      <c r="BE13" t="inlineStr"/>
-      <c r="BF13" t="inlineStr"/>
+      <c r="BD13" t="inlineStr">
+        <is>
+          <t>Strategic developments</t>
+        </is>
+      </c>
+      <c r="BE13" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="BF13" t="inlineStr">
+        <is>
+          <t>Government of Afghanistan (2021-)</t>
+        </is>
+      </c>
       <c r="BG13" t="inlineStr"/>
-      <c r="BH13" t="inlineStr"/>
-      <c r="BI13" t="inlineStr"/>
-      <c r="BJ13" t="inlineStr"/>
-      <c r="BK13" t="inlineStr"/>
-      <c r="BL13" t="n">
+      <c r="BH13" t="inlineStr">
+        <is>
+          <t>Civilians (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BI13" t="inlineStr">
+        <is>
+          <t>Students (Afghanistan); Teachers (Afghanistan); Women (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BJ13" t="inlineStr">
+        <is>
+          <t>Other: Around 12 May 2025 (as reported), the Taliban shut down 267 local education classes for girls in Paktika province (coded to Sharan), transferring the equipment to religious schools. This action has deprived 11,800 girls of education and left hundreds of teachers unemployed. The classes, supported by the WAIFA organization, were operating in remote areas lacking formal schools. Taliban have already barred girls above the sixth grade from attending school and closed universities to female students.</t>
+        </is>
+      </c>
+      <c r="BK13" t="inlineStr">
+        <is>
+          <t>2025-05-12</t>
+        </is>
+      </c>
+      <c r="BL13" t="inlineStr"/>
+      <c r="BM13" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2189,20 +2976,61 @@
       <c r="AV14" t="inlineStr"/>
       <c r="AW14" t="inlineStr"/>
       <c r="AX14" t="inlineStr"/>
-      <c r="AY14" t="inlineStr"/>
-      <c r="AZ14" t="inlineStr"/>
-      <c r="BA14" t="inlineStr"/>
-      <c r="BB14" t="inlineStr"/>
+      <c r="AY14" t="inlineStr">
+        <is>
+          <t>Paktia</t>
+        </is>
+      </c>
+      <c r="AZ14" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA14" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB14" t="inlineStr">
+        <is>
+          <t>AF1306</t>
+        </is>
+      </c>
       <c r="BC14" t="inlineStr"/>
-      <c r="BD14" t="inlineStr"/>
-      <c r="BE14" t="inlineStr"/>
-      <c r="BF14" t="inlineStr"/>
-      <c r="BG14" t="inlineStr"/>
-      <c r="BH14" t="inlineStr"/>
+      <c r="BD14" t="inlineStr">
+        <is>
+          <t>Protests</t>
+        </is>
+      </c>
+      <c r="BE14" t="inlineStr">
+        <is>
+          <t>Protest with intervention</t>
+        </is>
+      </c>
+      <c r="BF14" t="inlineStr">
+        <is>
+          <t>Protesters (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BG14" t="inlineStr">
+        <is>
+          <t>Civilians (Afghanistan); Students (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BH14" t="inlineStr">
+        <is>
+          <t>Military Forces of Afghanistan (2021-)</t>
+        </is>
+      </c>
       <c r="BI14" t="inlineStr"/>
-      <c r="BJ14" t="inlineStr"/>
-      <c r="BK14" t="inlineStr"/>
-      <c r="BL14" t="n">
+      <c r="BJ14" t="inlineStr">
+        <is>
+          <t>On 9 December 2024, hundreds of newly graduated students held a protest in front of the district headquarters in Sayyid Karam district, Paktia, after the Taliban collected 1,000 Afghanis from each student for a graduation ceremony. The Taliban district education director later prohibited it. The protesters were severely beaten and 'tortured' by the Taliban, leaving several injured, with some students transferred to unknown locations.</t>
+        </is>
+      </c>
+      <c r="BK14" t="inlineStr">
+        <is>
+          <t>2024-12-09</t>
+        </is>
+      </c>
+      <c r="BL14" t="inlineStr"/>
+      <c r="BM14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2274,47 +3102,150 @@
       <c r="W15" t="n">
         <v>25.88</v>
       </c>
-      <c r="X15" t="inlineStr"/>
-      <c r="Y15" t="inlineStr"/>
-      <c r="Z15" t="inlineStr"/>
-      <c r="AA15" t="inlineStr"/>
-      <c r="AB15" t="inlineStr"/>
-      <c r="AC15" t="inlineStr"/>
-      <c r="AD15" t="inlineStr"/>
-      <c r="AE15" t="inlineStr"/>
-      <c r="AF15" t="inlineStr"/>
-      <c r="AG15" t="inlineStr"/>
-      <c r="AH15" t="inlineStr"/>
-      <c r="AI15" t="inlineStr"/>
-      <c r="AJ15" t="inlineStr"/>
-      <c r="AK15" t="inlineStr"/>
-      <c r="AL15" t="inlineStr"/>
-      <c r="AM15" t="inlineStr"/>
-      <c r="AN15" t="inlineStr"/>
-      <c r="AO15" t="inlineStr"/>
-      <c r="AP15" t="inlineStr"/>
-      <c r="AQ15" t="inlineStr"/>
-      <c r="AR15" t="inlineStr"/>
-      <c r="AS15" t="inlineStr"/>
-      <c r="AT15" t="inlineStr"/>
-      <c r="AU15" t="inlineStr"/>
+      <c r="X15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO15" t="inlineStr">
+        <is>
+          <t>2025-05-21</t>
+        </is>
+      </c>
+      <c r="AP15" t="inlineStr">
+        <is>
+          <t>May 2025: An education facility was closed by the Taliban. Students and staff were forced to attend a seminar aimed at attracting youth to the Taliban.</t>
+        </is>
+      </c>
+      <c r="AQ15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Education Building </t>
+        </is>
+      </c>
+      <c r="AR15" t="inlineStr">
+        <is>
+          <t>Police</t>
+        </is>
+      </c>
+      <c r="AS15" t="inlineStr">
+        <is>
+          <t>Islamic Emirate of Afghanistan</t>
+        </is>
+      </c>
+      <c r="AT15" t="inlineStr">
+        <is>
+          <t>Firearms</t>
+        </is>
+      </c>
+      <c r="AU15" t="inlineStr">
+        <is>
+          <t>University</t>
+        </is>
+      </c>
       <c r="AV15" t="inlineStr"/>
       <c r="AW15" t="inlineStr"/>
       <c r="AX15" t="inlineStr"/>
-      <c r="AY15" t="inlineStr"/>
-      <c r="AZ15" t="inlineStr"/>
-      <c r="BA15" t="inlineStr"/>
-      <c r="BB15" t="inlineStr"/>
+      <c r="AY15" t="inlineStr">
+        <is>
+          <t>Khost</t>
+        </is>
+      </c>
+      <c r="AZ15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA15" t="n">
+        <v>6</v>
+      </c>
+      <c r="BB15" t="inlineStr">
+        <is>
+          <t>AF1401</t>
+        </is>
+      </c>
       <c r="BC15" t="inlineStr"/>
-      <c r="BD15" t="inlineStr"/>
-      <c r="BE15" t="inlineStr"/>
-      <c r="BF15" t="inlineStr"/>
+      <c r="BD15" t="inlineStr">
+        <is>
+          <t>Strategic developments ---- Strategic developments ---- Strategic developments ---- Violence against civilians ---- Strategic developments ---- Strategic developments</t>
+        </is>
+      </c>
+      <c r="BE15" t="inlineStr">
+        <is>
+          <t>Other ---- Other ---- Other ---- Attack ---- Other ---- Other</t>
+        </is>
+      </c>
+      <c r="BF15" t="inlineStr">
+        <is>
+          <t>Government of Afghanistan (2021-) ---- Government of Afghanistan (2021-) ---- Government of Afghanistan (2021-) ---- Military Forces of Afghanistan (2021-) ---- Government of Afghanistan (2021-) ---- Government of Afghanistan (2021-)</t>
+        </is>
+      </c>
       <c r="BG15" t="inlineStr"/>
-      <c r="BH15" t="inlineStr"/>
-      <c r="BI15" t="inlineStr"/>
-      <c r="BJ15" t="inlineStr"/>
-      <c r="BK15" t="inlineStr"/>
-      <c r="BL15" t="n">
+      <c r="BH15" t="inlineStr">
+        <is>
+          <t>Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BI15" t="inlineStr">
+        <is>
+          <t>Journalists (Afghanistan) ---- Students (Afghanistan); Journalists (Afghanistan) ---- Prisoners (Afghanistan); Teachers (Afghanistan) ---- Students (Afghanistan) ---- Teachers (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BJ15" t="inlineStr">
+        <is>
+          <t>Other: On 24 August 2024, The Taliban Ministry of Education ordered local media in Khost province to halt the publication of educational programs for school subjects above the sixth grade, warning that they will face punishment for any violations. This educational programs benefited many girls above sixth grade who were prohibited from attending schools by Taliban order. ---- Other: On 19 October 2024, the Taliban's Higher Education Minister prohibited journalists from filming or creating any visual documentation at an event held at Sheikh Zayed University in Khost province. Journalists were only allowed to prepare written reports of the meeting. This ban was implemented under the Taliban's new 'Vice and Virtue' law, which prohibited the publication of images of living beings. ---- Other: Around 3 November 2024 (as reported), the Taliban banned journalism students at Sheikh Zayed University in Khost province from taking pictures or filming, warning that those who disobeyed the order would face punishment. The students expressed that the new ban created serious challenges for their practical work. This ban was enforced under the Taliban's new 'Vice and Virtue' law, which prohibits the publication of images of living beings. ---- Around 3 December 2024 (as reported), bodyguards of the Taliban governor in Khost province severely beat a professor from the Faculty of Jurisprudence at Sheikh Zayed University, causing him to faint. He was then transferred to the governor's private prison, where he is being tortured. The incident followed the professor's opposition to the governor's representatives sent to evaluate the university's professors. Sources said that the Taliban governor intends to dismiss the current professors of the Faculty of Jurisprudence and replace them with graduates from religious schools. ---- Other: Around 17 December 2024 (as reported), Taliban Education Department in Khost province declared 130 newly graduated 12th-grade students as failed. The decision was made because the students wrote commemorative signatures and autographs on each other's uniforms during their graduation ceremony, which the Taliban claimed was against Islamic laws. ---- Other: Around 6 March 2025 (as reported), the Taliban dismissed numerous teachers in Khost city, replacing them with graduates of religious schools. The dismissals were due to teachers trimming their beards and failing to comply with Taliban regulations. 40 teachers from Mohammad Sadiq High School and more than 10 professors from Sheikh Zayed University were among those removed from their positions.</t>
+        </is>
+      </c>
+      <c r="BK15" t="inlineStr">
+        <is>
+          <t>2024-08-24 ---- 2024-10-19 ---- 2024-11-03 ---- 2024-12-03 ---- 2024-12-17 ---- 2025-03-06</t>
+        </is>
+      </c>
+      <c r="BL15" t="inlineStr"/>
+      <c r="BM15" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2413,20 +3344,61 @@
       <c r="AV16" t="inlineStr"/>
       <c r="AW16" t="inlineStr"/>
       <c r="AX16" t="inlineStr"/>
-      <c r="AY16" t="inlineStr"/>
-      <c r="AZ16" t="inlineStr"/>
-      <c r="BA16" t="inlineStr"/>
-      <c r="BB16" t="inlineStr"/>
+      <c r="AY16" t="inlineStr">
+        <is>
+          <t>Kunar</t>
+        </is>
+      </c>
+      <c r="AZ16" t="n">
+        <v>2</v>
+      </c>
+      <c r="BA16" t="n">
+        <v>5</v>
+      </c>
+      <c r="BB16" t="inlineStr">
+        <is>
+          <t>AF1501</t>
+        </is>
+      </c>
       <c r="BC16" t="inlineStr"/>
-      <c r="BD16" t="inlineStr"/>
-      <c r="BE16" t="inlineStr"/>
-      <c r="BF16" t="inlineStr"/>
+      <c r="BD16" t="inlineStr">
+        <is>
+          <t>Violence against civilians ---- Strategic developments ---- Strategic developments ---- Violence against civilians ---- Strategic developments</t>
+        </is>
+      </c>
+      <c r="BE16" t="inlineStr">
+        <is>
+          <t>Attack ---- Other ---- Other ---- Attack ---- Other</t>
+        </is>
+      </c>
+      <c r="BF16" t="inlineStr">
+        <is>
+          <t>Police Forces of Afghanistan (2021-) General Directorate of Intelligence ---- Government of Afghanistan (2021-) ---- Government of Afghanistan (2021-) ---- Military Forces of Afghanistan (2021-) ---- Government of Afghanistan (2021-)</t>
+        </is>
+      </c>
       <c r="BG16" t="inlineStr"/>
-      <c r="BH16" t="inlineStr"/>
-      <c r="BI16" t="inlineStr"/>
-      <c r="BJ16" t="inlineStr"/>
-      <c r="BK16" t="inlineStr"/>
-      <c r="BL16" t="n">
+      <c r="BH16" t="inlineStr">
+        <is>
+          <t>Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BI16" t="inlineStr">
+        <is>
+          <t>Muslim Group (Afghanistan); Prisoners (Afghanistan); Salafist Muslim Group (Afghanistan); Teachers (Afghanistan) ---- Journalists (Afghanistan) ---- Salafist Muslim Group (Afghanistan) ---- Health Workers (Afghanistan); Students (Afghanistan) ---- Students (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BJ16" t="inlineStr">
+        <is>
+          <t>Around 13 May 2024 (month of), Salafi religious scholar was arrested by Taliban intelligence forces in Asad Abad city, Kunar, over alleged links to IS. He was severely tortured in a Taliban prison in Kabul. He was teaching at a religious school in Asadabad. ---- Other: Around 4 November 2024 (as reported), the Taliban's Higher Education Minister prohibited journalists from photographing or filming during his meeting with students and officials at Syed Jamaluddin Afghan University in Asad Abad city (Kunar), expelling them from the event. Only audio media reporters were allowed to cover the meeting. This restriction was imposed under the Taliban's new 'Vice and Virtue' law, which bans the publication of images of living beings. ---- Other: On 1 January 2025, the Taliban closed Salafi schools in Asad Abad city, Kunar, claiming that these institutions were promoting IS ideology among the youth. ---- On 31 March 2025, two men were killed by Taliban members in the Shin Koruk Darah village of Shigal district, Kunar. The two men were engaged in a dispute and Taliban fired at them as they were trying to control the situation. The Taliban members were visiting the province. A religious scholar from Kunar asked the Taliban to punish the killers. One of the deceased was a final-year medical student studying abroad. ---- Other: On 5 August 2025, the Taliban's Ministry for the Promotion of Virtue and Prevention of Vice banned photography of university graduation ceremonies in Kunar province (coded to Asad Abad). This restriction was imposed under the Taliban's new 'Vice and Virtue' law, which prohibits the publication of images of living beings.</t>
+        </is>
+      </c>
+      <c r="BK16" t="inlineStr">
+        <is>
+          <t>2024-05-13 ---- 2024-11-04 ---- 2025-01-01 ---- 2025-03-31 ---- 2025-08-05</t>
+        </is>
+      </c>
+      <c r="BL16" t="inlineStr"/>
+      <c r="BM16" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2525,20 +3497,61 @@
       <c r="AV17" t="inlineStr"/>
       <c r="AW17" t="inlineStr"/>
       <c r="AX17" t="inlineStr"/>
-      <c r="AY17" t="inlineStr"/>
-      <c r="AZ17" t="inlineStr"/>
-      <c r="BA17" t="inlineStr"/>
-      <c r="BB17" t="inlineStr"/>
+      <c r="AY17" t="inlineStr">
+        <is>
+          <t>Nuristan</t>
+        </is>
+      </c>
+      <c r="AZ17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA17" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB17" t="inlineStr">
+        <is>
+          <t>AF1601</t>
+        </is>
+      </c>
       <c r="BC17" t="inlineStr"/>
-      <c r="BD17" t="inlineStr"/>
-      <c r="BE17" t="inlineStr"/>
-      <c r="BF17" t="inlineStr"/>
+      <c r="BD17" t="inlineStr">
+        <is>
+          <t>Strategic developments</t>
+        </is>
+      </c>
+      <c r="BE17" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="BF17" t="inlineStr">
+        <is>
+          <t>Government of Afghanistan (2021-)</t>
+        </is>
+      </c>
       <c r="BG17" t="inlineStr"/>
-      <c r="BH17" t="inlineStr"/>
-      <c r="BI17" t="inlineStr"/>
-      <c r="BJ17" t="inlineStr"/>
-      <c r="BK17" t="inlineStr"/>
-      <c r="BL17" t="n">
+      <c r="BH17" t="inlineStr">
+        <is>
+          <t>Civilians (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BI17" t="inlineStr">
+        <is>
+          <t>Journalists (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BJ17" t="inlineStr">
+        <is>
+          <t>Other: On 2 November 2024, the Taliban's Higher Education Minister prohibited journalists from filming or photographing a meeting in Nuristan (coded to Paroon) province and expelled them from the event. Only audio media reporters were permitted to cover the meeting. This restriction was enforced under the Taliban's new 'Vice and Virtue' law, which bans the publication of images of living beings.</t>
+        </is>
+      </c>
+      <c r="BK17" t="inlineStr">
+        <is>
+          <t>2024-11-02</t>
+        </is>
+      </c>
+      <c r="BL17" t="inlineStr"/>
+      <c r="BM17" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2610,47 +3623,150 @@
       <c r="W18" t="n">
         <v>31.61</v>
       </c>
-      <c r="X18" t="inlineStr"/>
-      <c r="Y18" t="inlineStr"/>
-      <c r="Z18" t="inlineStr"/>
-      <c r="AA18" t="inlineStr"/>
-      <c r="AB18" t="inlineStr"/>
-      <c r="AC18" t="inlineStr"/>
-      <c r="AD18" t="inlineStr"/>
-      <c r="AE18" t="inlineStr"/>
-      <c r="AF18" t="inlineStr"/>
-      <c r="AG18" t="inlineStr"/>
-      <c r="AH18" t="inlineStr"/>
-      <c r="AI18" t="inlineStr"/>
-      <c r="AJ18" t="inlineStr"/>
-      <c r="AK18" t="inlineStr"/>
-      <c r="AL18" t="inlineStr"/>
-      <c r="AM18" t="inlineStr"/>
-      <c r="AN18" t="inlineStr"/>
-      <c r="AO18" t="inlineStr"/>
-      <c r="AP18" t="inlineStr"/>
-      <c r="AQ18" t="inlineStr"/>
-      <c r="AR18" t="inlineStr"/>
-      <c r="AS18" t="inlineStr"/>
-      <c r="AT18" t="inlineStr"/>
-      <c r="AU18" t="inlineStr"/>
+      <c r="X18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN18" t="n">
+        <v>2</v>
+      </c>
+      <c r="AO18" t="inlineStr">
+        <is>
+          <t>2024-09-03 ---- 2024-08-08</t>
+        </is>
+      </c>
+      <c r="AP18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">September 2024: A teacher was shot and killed by the Taliban's district education chief. Some sources reported that the teacher was supposed to be appointed as the district‚Äôs new education chief and was killed due to this.  ---- August 2024: A educator was beaten by a Taliban mayor for posting a critical article on social media about the mayor's usurpation of people's shops and lands. </t>
+        </is>
+      </c>
+      <c r="AQ18" t="inlineStr">
+        <is>
+          <t>Unspecified Location ---- Unspecified Location</t>
+        </is>
+      </c>
+      <c r="AR18" t="inlineStr">
+        <is>
+          <t>Other ---- Other</t>
+        </is>
+      </c>
+      <c r="AS18" t="inlineStr">
+        <is>
+          <t>Islamic Emirate of Afghanistan ---- Islamic Emirate of Afghanistan</t>
+        </is>
+      </c>
+      <c r="AT18" t="inlineStr">
+        <is>
+          <t>Firearms ---- Fist and Foot</t>
+        </is>
+      </c>
+      <c r="AU18" t="inlineStr">
+        <is>
+          <t>Not Applicable ---- Not Applicable</t>
+        </is>
+      </c>
       <c r="AV18" t="inlineStr"/>
       <c r="AW18" t="inlineStr"/>
       <c r="AX18" t="inlineStr"/>
-      <c r="AY18" t="inlineStr"/>
-      <c r="AZ18" t="inlineStr"/>
-      <c r="BA18" t="inlineStr"/>
-      <c r="BB18" t="inlineStr"/>
+      <c r="AY18" t="inlineStr">
+        <is>
+          <t>Badakhshan</t>
+        </is>
+      </c>
+      <c r="AZ18" t="n">
+        <v>3</v>
+      </c>
+      <c r="BA18" t="n">
+        <v>11</v>
+      </c>
+      <c r="BB18" t="inlineStr">
+        <is>
+          <t>AF1701</t>
+        </is>
+      </c>
       <c r="BC18" t="inlineStr"/>
-      <c r="BD18" t="inlineStr"/>
-      <c r="BE18" t="inlineStr"/>
-      <c r="BF18" t="inlineStr"/>
+      <c r="BD18" t="inlineStr">
+        <is>
+          <t>Strategic developments ---- Violence against civilians ---- Strategic developments ---- Violence against civilians ---- Violence against civilians ---- Violence against civilians ---- Violence against civilians ---- Violence against civilians ---- Violence against civilians ---- Strategic developments ---- Strategic developments</t>
+        </is>
+      </c>
+      <c r="BE18" t="inlineStr">
+        <is>
+          <t>Other ---- Sexual violence ---- Other ---- Attack ---- Attack ---- Abduction/forced disappearance ---- Attack ---- Sexual violence ---- Attack ---- Other ---- Other</t>
+        </is>
+      </c>
+      <c r="BF18" t="inlineStr">
+        <is>
+          <t>Military Forces of Afghanistan (2021-) ---- Military Forces of Afghanistan (2021-) ---- Military Forces of Afghanistan (2021-) ---- Military Forces of Afghanistan (2021-) ---- Military Forces of Afghanistan (2021-) ---- Military Forces of Afghanistan (2021-) ---- Military Forces of Afghanistan (2021-) ---- Military Forces of Afghanistan (2021-) ---- Military Forces of Afghanistan (2021-) ---- Government of Afghanistan (2021-) ---- Government of Afghanistan (2021-)</t>
+        </is>
+      </c>
       <c r="BG18" t="inlineStr"/>
-      <c r="BH18" t="inlineStr"/>
-      <c r="BI18" t="inlineStr"/>
-      <c r="BJ18" t="inlineStr"/>
-      <c r="BK18" t="inlineStr"/>
-      <c r="BL18" t="n">
+      <c r="BH18" t="inlineStr">
+        <is>
+          <t>Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BI18" t="inlineStr">
+        <is>
+          <t>Ismaili Muslim Group (Afghanistan) ---- Students (Afghanistan); Women (Afghanistan) ---- Teachers (Afghanistan) ---- Teachers (Afghanistan) ---- Students (Afghanistan); Women (Afghanistan) ---- Labor Group (Afghanistan) ---- Students (Afghanistan); Women (Afghanistan) ---- Ismaili Muslim Group (Afghanistan); Students (Afghanistan) ---- Women (Afghanistan); Students (Afghanistan) ---- Salafist Muslim Group (Afghanistan); Teachers (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BJ18" t="inlineStr">
+        <is>
+          <t>Other: Around 23 January 2024 (as reported), the Taliban established tens of Sunni religious schools in Eshkashim, Shighnan, Yamgan, and Zebak (all coded to Faiz Abad), Badakhshan, and warned the Ismaili Muslim residents to enroll their children in the Sunni religious schools to change their religion. Approximately 600 Ismaili children were recruited, and Ismaili Muslims were prohibited from attending their own religious congregations. ---- Around 23 January 2024, the head of a religious girls school, a Taliban member, raped a 17 year-old student in the Dasht Qarugh area of Faiz Abad city, Badakhshan. The girl became pregnant. He got arrested after a complaint by the girl's family. He was reported to be married to four women, two of whom were students at the same school. He ran away before he got arrested. ---- Other: Around 15 June 2024 (as reported), Taliban district governor recruited at least 30 children aged 10 to 18 from religious schools to special military training center and provided them with training despite the opposition of the parents, in Tarbiya Moalem area of Nesay district [coded to Jamarj-e Bala], Badakhshan. ---- On 8 August 2024, Taliban's mayor of Badakhshan called a teacher to his office in Faiz Abad city, Badakhshan and severely beat him for posting a critical article on Facebook about the mayor's usurpation of people's shops and lands. ---- Around 3 September 2024, a teacher was shot and killed by the Taliban's district education chief in the center of Eshkashim district, Badakhshan. Some sources claimed that the teacher was supposed to be appointed as the new education chief for the district and was killed due to this. ---- Around 1 November 2024 (beginning of month), a young female student was abducted by suspected Taliban members in Faiz Abad city, Badakhshan, after receiving a phone call asking her to bring a book to her religious school. She was subsequently gang-raped and killed (coded separately), and her body was discovered 14 days later by locals along the riverbank. ---- On 12 November 2024, the Taliban beat and dismissed the manager of the Badakhshan University dormitory in Faiz Abad city, Badakhshan, for refusing to grant dormitory accommodations to some Pashtun students. ---- Around 15 November 2024 (as reported), a young female student was gang-raped and killed by suspected Taliban members in Faiz Abad city, Badakhshan, before her body was thrown into a river. According to her family, she had received a phone call asking her to bring a book to her religious school, after which she was abducted (coded separately). Her body was discovered 14 days later by locals along the riverbank. ---- On 15 December 2024, an Ismaili boy, who was a seventh-grade student, was shot and killed by Taliban forces in Dugurgunt (Digargand) village of Wakhan district, Badakhshan. Motive unknown. The Taliban claimed the shooting was a mistake and stated that two individuals had been arrested in connection with the incident. ---- Other: On 14 January 2025, the Taliban shut down education centers, English language institutes, and kindergartens for girls below the sixth grade in Faiz Abad city, Badakhshan. These institutions were supported by the Agha Khan Foundation. ---- Other: Around 10 March 2025 (as reported), the Taliban Ministry of Higher Education dismissed six professors from the Faculty of Sharia at the university in Badakhshan (coded to Faiz Abad) province. Sources said that they were dismissed due to their Salafi beliefs. The dismissed professors held high academic degrees and had more than ten years of teaching experience.</t>
+        </is>
+      </c>
+      <c r="BK18" t="inlineStr">
+        <is>
+          <t>2024-01-23 ---- 2024-01-23 ---- 2024-06-15 ---- 2024-08-08 ---- 2024-09-03 ---- 2024-11-01 ---- 2024-11-12 ---- 2024-11-15 ---- 2024-12-15 ---- 2025-01-14 ---- 2025-03-10</t>
+        </is>
+      </c>
+      <c r="BL18" t="inlineStr"/>
+      <c r="BM18" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2722,47 +3838,154 @@
       <c r="W19" t="n">
         <v>42.44</v>
       </c>
-      <c r="X19" t="inlineStr"/>
-      <c r="Y19" t="inlineStr"/>
-      <c r="Z19" t="inlineStr"/>
-      <c r="AA19" t="inlineStr"/>
-      <c r="AB19" t="inlineStr"/>
-      <c r="AC19" t="inlineStr"/>
-      <c r="AD19" t="inlineStr"/>
-      <c r="AE19" t="inlineStr"/>
-      <c r="AF19" t="inlineStr"/>
-      <c r="AG19" t="inlineStr"/>
-      <c r="AH19" t="inlineStr"/>
-      <c r="AI19" t="inlineStr"/>
-      <c r="AJ19" t="inlineStr"/>
-      <c r="AK19" t="inlineStr"/>
-      <c r="AL19" t="inlineStr"/>
-      <c r="AM19" t="inlineStr"/>
-      <c r="AN19" t="inlineStr"/>
-      <c r="AO19" t="inlineStr"/>
-      <c r="AP19" t="inlineStr"/>
-      <c r="AQ19" t="inlineStr"/>
-      <c r="AR19" t="inlineStr"/>
-      <c r="AS19" t="inlineStr"/>
-      <c r="AT19" t="inlineStr"/>
-      <c r="AU19" t="inlineStr"/>
+      <c r="X19" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH19" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN19" t="n">
+        <v>2</v>
+      </c>
+      <c r="AO19" t="inlineStr">
+        <is>
+          <t>2024-10-13 ---- 2024-02-25</t>
+        </is>
+      </c>
+      <c r="AP19" t="inlineStr">
+        <is>
+          <t>October 2024: A male student was beaten, shot and killed by a Taliban fighter near a school.  ---- February 2024: a school guard was injured and educational materials looted in a nighttime attack on a school by unidentified armed men.</t>
+        </is>
+      </c>
+      <c r="AQ19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Education Building  ---- Education Building </t>
+        </is>
+      </c>
+      <c r="AR19" t="inlineStr">
+        <is>
+          <t>Police ---- NSA</t>
+        </is>
+      </c>
+      <c r="AS19" t="inlineStr">
+        <is>
+          <t>Islamic Emirate of Afghanistan ---- Unidentified Armed Actor</t>
+        </is>
+      </c>
+      <c r="AT19" t="inlineStr">
+        <is>
+          <t>Firearms ---- Firearms</t>
+        </is>
+      </c>
+      <c r="AU19" t="inlineStr">
+        <is>
+          <t>Secondary School ---- School: No Further Details</t>
+        </is>
+      </c>
       <c r="AV19" t="inlineStr"/>
       <c r="AW19" t="inlineStr"/>
       <c r="AX19" t="inlineStr"/>
-      <c r="AY19" t="inlineStr"/>
-      <c r="AZ19" t="inlineStr"/>
-      <c r="BA19" t="inlineStr"/>
-      <c r="BB19" t="inlineStr"/>
+      <c r="AY19" t="inlineStr">
+        <is>
+          <t>Takhar</t>
+        </is>
+      </c>
+      <c r="AZ19" t="n">
+        <v>5</v>
+      </c>
+      <c r="BA19" t="n">
+        <v>15</v>
+      </c>
+      <c r="BB19" t="inlineStr">
+        <is>
+          <t>AF1801</t>
+        </is>
+      </c>
       <c r="BC19" t="inlineStr"/>
-      <c r="BD19" t="inlineStr"/>
-      <c r="BE19" t="inlineStr"/>
-      <c r="BF19" t="inlineStr"/>
-      <c r="BG19" t="inlineStr"/>
-      <c r="BH19" t="inlineStr"/>
-      <c r="BI19" t="inlineStr"/>
-      <c r="BJ19" t="inlineStr"/>
-      <c r="BK19" t="inlineStr"/>
-      <c r="BL19" t="n">
+      <c r="BD19" t="inlineStr">
+        <is>
+          <t>Strategic developments ---- Strategic developments ---- Violence against civilians ---- Violence against civilians ---- Strategic developments ---- Violence against civilians ---- Violence against civilians ---- Explosions/Remote violence ---- Violence against civilians ---- Protests ---- Violence against civilians ---- Violence against civilians ---- Violence against civilians ---- Protests ---- Battles</t>
+        </is>
+      </c>
+      <c r="BE19" t="inlineStr">
+        <is>
+          <t>Arrests ---- Arrests ---- Attack ---- Sexual violence ---- Other ---- Abduction/forced disappearance ---- Sexual violence ---- Remote explosive/landmine/IED ---- Attack ---- Peaceful protest ---- Attack ---- Attack ---- Attack ---- Protest with intervention ---- Armed clash</t>
+        </is>
+      </c>
+      <c r="BF19" t="inlineStr">
+        <is>
+          <t>Police Forces of Afghanistan (2021-) General Directorate of Intelligence ---- Police Forces of Afghanistan (2021-) General Directorate of Intelligence ---- Unidentified Armed Group (Afghanistan) ---- Military Forces of Afghanistan (2021-) ---- Government of Afghanistan (2021-) ---- Police Forces of Afghanistan (2021-) General Directorate of Intelligence ---- Military Forces of Afghanistan (2021-) ---- National Resistance Front ---- Military Forces of Afghanistan (2021-) ---- Protesters (Afghanistan) ---- Unidentified Armed Group (Afghanistan) ---- Unidentified Armed Group (Afghanistan) ---- Military Forces of Afghanistan (2021-) ---- Protesters (Afghanistan) ---- National Resistance Front</t>
+        </is>
+      </c>
+      <c r="BG19" t="inlineStr">
+        <is>
+          <t>Purple Saturdays Movement; Women (Afghanistan) ---- Health Workers (Afghanistan); Students (Afghanistan); Women (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BH19" t="inlineStr">
+        <is>
+          <t>Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Military Forces of Afghanistan (2021-) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Police Forces of Afghanistan (2021-) General Directorate of Intelligence ---- Military Forces of Afghanistan (2021-)</t>
+        </is>
+      </c>
+      <c r="BI19" t="inlineStr">
+        <is>
+          <t>Hizb ut-Tahrir; Students (Afghanistan); Teachers (Afghanistan) ---- Hizb ut-Tahrir; Students (Afghanistan); Teachers (Afghanistan) ---- Labor Group (Afghanistan) ---- Prisoners (Afghanistan); Students (Afghanistan); Women (Afghanistan) ---- Students (Afghanistan); Women (Afghanistan) ---- Men (Afghanistan) ---- Civilians (Afghanistan) ---- Labor Group (Afghanistan); Students (Afghanistan) ---- Muslim Group (Afghanistan); Teachers (Afghanistan) ---- Former Military Forces of Afghanistan (2021-); Labor Group (Afghanistan) ---- Teachers (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BJ19" t="inlineStr">
+        <is>
+          <t>On 13 January 2024, Taliban intelligence forces apprehended approximately 15-16 members of Hizb-ut-Tahrir, including teachers and students, from a residential house in PD2 area of Taluqan city, Takhar. The individuals were carrying propaganda banners of Hizb Tahrir while they were arrested by the Taliban. ---- On 14 January 2024, Taliban intelligence forces arrested nine people including of teachers and students, suspected of having Hizb-ut-Tahrir membership from a guest house in Tagab-e Mian Shahr area of Warsaj district, Takhar. ---- On 25 February 2024, unidentified armed men attacked 'Khaja Changhan' boy's school near a Taliban security outpost in Chanzi village of Taluqan city, Takhar, leaving the school's guard severely injured and looted all supplies of the school. The motive and identities of the attackers remained undisclosed. Attack took place during the night. ---- Around 20 March 2024, a female protester and student was arrested by the Taliban at a checkpoint in PD6 of Taluqan city, Takhar, and was raped by a Taliban member while in prison. She had previously participated in 8 March protest against the Taliban. Her father later paid 60,000 Afghanis for her release, after which she was forced into marrying a 50-year-old man. ---- Other: On 2 June 2024, Taliban ordered the closure of all Darul Uloom and Darul Hafaz (religious schools known as madrassas) for teaching girls above the 10th grade in Taluqan city, Takhar. Girls enrolled in these schools after Taliban's nation-wide ban on girls education (coded separately). ---- On 15 August 2024, Taliban intelligence forces arrested the brother of a female protester and women's rights activist, who leads the Takhar Women's Movement and the Hooshmand Online School, in Taluqan city, Takhar. She claimed that her brother remains in Taliban intelligence custody with no information about his condition, and that the Taliban demanded property documents of four shops and a guarantee from 50 people to secure his release. She, now living abroad, had been arrested for protesting against the Taliban's restrictions on women (coded separately). ---- On 16 August 2024, Taliban forces based at Sherah School gang raped a 12-year-old male child in the Sherah Chi area of Eshkamesh district, Takhar. The child has been hospitalized in critical condition. ---- On 5 October 2024, an explosion occurred in front of the Molla Abdul Wadud Shahid High School in Taluqan city, Takhar, injuring 3-5 civilians, including children. NRF sources took responsibility for the attack, claiming that the head of logistics of the Taliban Ministry of Interior along with one of his companions were killed, and another Taliban member was wounded. However, health sources in Takhar claimed that the Taliban's logistics head was severely wounded, not killed. ---- On 13 October 2024, a Taliban fighter beat and then shot dead a young boy following a verbal dispute near Abu Osmani Taleghani high school in Taluqan city, Takhar. The victim was a student who also worked as a service employee in a building. The reason for the dispute remained unknown. ---- On 19 October 2024, a group of women from the 'Purple Saturdays Movement' held an indoor protest in Taluqan city, Takhar. They stated that the closure of girls' schools represents a significant disaster for Afghanistan, as more than half of the population is deprived of the right to education, however, that the reopening of girls' schools under Taliban rule is even more disastrous, as it promotes extremist ideology and doctrines. ---- On 1 November 2024, a religious scholar and school teacher was killed by unknown gunmen in the Nowabad Moshtaniha area of Taluqan city, Takhar, while on his way to morning prayer. The motive remains unclear. He had occasionally criticized Taliban policies and advocated for women's education. ---- On 7 November 2024, a former security officer was hanged by unknown attackers inside a school building in Taluqan city, Takhar. Motive unknown. Following the Taliban takeover, he had been working as a driver for a private school. ---- On 18 November 2024, two Taliban guards severely beat an administrator of Takhar University in Taluqan city, Takhar, over lack of food. No further information. ---- Around 3 December 2024 (as reported), a number of female students from medical institutes protested in Takhar province (coded to Taluqan) against the Taliban's order to cease female education in all public and private medical institutes (coded separately). At least two female students were arrested by Taliban intelligence, with reports that several others were arrested. ---- On 14 February 2025, a clash erupted between National Resistance Front militants and Taliban forces following an explosion carried out by NRF at a security outpost of the Taliban Statistics Department near Dr. Hussein Shaheed School in Taluqan city, Takhar. Two Taliban members were killed, another was wounded, and a Taliban vehicle was also destroyed. No casualties from NRF. Local sources confirmed hearing both an explosion and subsequent gunfire.</t>
+        </is>
+      </c>
+      <c r="BK19" t="inlineStr">
+        <is>
+          <t>2024-01-13 ---- 2024-01-14 ---- 2024-02-25 ---- 2024-03-20 ---- 2024-06-02 ---- 2024-08-15 ---- 2024-08-16 ---- 2024-10-05 ---- 2024-10-13 ---- 2024-10-19 ---- 2024-11-01 ---- 2024-11-07 ---- 2024-11-18 ---- 2024-12-03 ---- 2025-02-14</t>
+        </is>
+      </c>
+      <c r="BL19" t="inlineStr"/>
+      <c r="BM19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2861,20 +4084,61 @@
       <c r="AV20" t="inlineStr"/>
       <c r="AW20" t="inlineStr"/>
       <c r="AX20" t="inlineStr"/>
-      <c r="AY20" t="inlineStr"/>
-      <c r="AZ20" t="inlineStr"/>
-      <c r="BA20" t="inlineStr"/>
-      <c r="BB20" t="inlineStr"/>
+      <c r="AY20" t="inlineStr">
+        <is>
+          <t>Kunduz</t>
+        </is>
+      </c>
+      <c r="AZ20" t="n">
+        <v>19</v>
+      </c>
+      <c r="BA20" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB20" t="inlineStr">
+        <is>
+          <t>AF1901</t>
+        </is>
+      </c>
       <c r="BC20" t="inlineStr"/>
-      <c r="BD20" t="inlineStr"/>
-      <c r="BE20" t="inlineStr"/>
-      <c r="BF20" t="inlineStr"/>
+      <c r="BD20" t="inlineStr">
+        <is>
+          <t>Explosions/Remote violence</t>
+        </is>
+      </c>
+      <c r="BE20" t="inlineStr">
+        <is>
+          <t>Suicide bomb</t>
+        </is>
+      </c>
+      <c r="BF20" t="inlineStr">
+        <is>
+          <t>Islamic State Khorasan Province (ISKP)</t>
+        </is>
+      </c>
       <c r="BG20" t="inlineStr"/>
-      <c r="BH20" t="inlineStr"/>
-      <c r="BI20" t="inlineStr"/>
-      <c r="BJ20" t="inlineStr"/>
-      <c r="BK20" t="inlineStr"/>
-      <c r="BL20" t="n">
+      <c r="BH20" t="inlineStr">
+        <is>
+          <t>Military Forces of Afghanistan (2021-)</t>
+        </is>
+      </c>
+      <c r="BI20" t="inlineStr">
+        <is>
+          <t>Labor Group (Afghanistan); Police Forces of Afghanistan (2021-); Teachers (Afghanistan); Civilians (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BJ20" t="inlineStr">
+        <is>
+          <t>On 11 February 2025, an IS suicide bomber detonated himself outside the Kabul Bank in Kunduz city, where Taliban members and civilians were waiting in line to receive salaries and withdraw money. There are varying reports on fatalities, 15-30 people, mostly Taliban defense ministry members, reported to have been killed and 14-40 wounded in the explosion. Among the killed were a bank guard, 8 Taliban army and police members, a Taliban security commander, and a university professor. The Taliban claimed that 8 people, including their members, bank guards, and civilians, were killed, with 7 others wounded, while the IS claimed that dozens of Taliban members, including security commanders, were killed and wounded in the attack. One Taliban member claimed that 20 Taliban members and 4 civilians were killed, with 12 others wounded in the attack. The bodies of 18 deceased were brought to a local medical facility. Prior to this attack, the Taliban had reportedly instructed their fighters not to visit Kabul Bank branches to collect their salaries. Fatalities coded as 19 based on bodies received at the local medical facility, and including the suicide bomber.</t>
+        </is>
+      </c>
+      <c r="BK20" t="inlineStr">
+        <is>
+          <t>2025-02-11</t>
+        </is>
+      </c>
+      <c r="BL20" t="inlineStr"/>
+      <c r="BM20" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2986,7 +4250,8 @@
       <c r="BI21" t="inlineStr"/>
       <c r="BJ21" t="inlineStr"/>
       <c r="BK21" t="inlineStr"/>
-      <c r="BL21" t="n">
+      <c r="BL21" t="inlineStr"/>
+      <c r="BM21" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3058,47 +4323,154 @@
       <c r="W22" t="n">
         <v>36.11</v>
       </c>
-      <c r="X22" t="inlineStr"/>
-      <c r="Y22" t="inlineStr"/>
-      <c r="Z22" t="inlineStr"/>
-      <c r="AA22" t="inlineStr"/>
-      <c r="AB22" t="inlineStr"/>
-      <c r="AC22" t="inlineStr"/>
-      <c r="AD22" t="inlineStr"/>
-      <c r="AE22" t="inlineStr"/>
-      <c r="AF22" t="inlineStr"/>
-      <c r="AG22" t="inlineStr"/>
-      <c r="AH22" t="inlineStr"/>
-      <c r="AI22" t="inlineStr"/>
-      <c r="AJ22" t="inlineStr"/>
-      <c r="AK22" t="inlineStr"/>
-      <c r="AL22" t="inlineStr"/>
-      <c r="AM22" t="inlineStr"/>
-      <c r="AN22" t="inlineStr"/>
-      <c r="AO22" t="inlineStr"/>
-      <c r="AP22" t="inlineStr"/>
-      <c r="AQ22" t="inlineStr"/>
-      <c r="AR22" t="inlineStr"/>
-      <c r="AS22" t="inlineStr"/>
-      <c r="AT22" t="inlineStr"/>
-      <c r="AU22" t="inlineStr"/>
+      <c r="X22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO22" t="inlineStr">
+        <is>
+          <t>2024-09-04</t>
+        </is>
+      </c>
+      <c r="AP22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">September 2024: A teacher was shot and killed by two gunmen riding a motorcycle. The men also stole the teacher‚Äôs cell phone. </t>
+        </is>
+      </c>
+      <c r="AQ22" t="inlineStr">
+        <is>
+          <t>Private Travel</t>
+        </is>
+      </c>
+      <c r="AR22" t="inlineStr">
+        <is>
+          <t>Criminal</t>
+        </is>
+      </c>
+      <c r="AS22" t="inlineStr">
+        <is>
+          <t>Unidentified Armed Actor</t>
+        </is>
+      </c>
+      <c r="AT22" t="inlineStr">
+        <is>
+          <t>Firearms</t>
+        </is>
+      </c>
+      <c r="AU22" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
       <c r="AV22" t="inlineStr"/>
       <c r="AW22" t="inlineStr"/>
       <c r="AX22" t="inlineStr"/>
-      <c r="AY22" t="inlineStr"/>
-      <c r="AZ22" t="inlineStr"/>
-      <c r="BA22" t="inlineStr"/>
-      <c r="BB22" t="inlineStr"/>
+      <c r="AY22" t="inlineStr">
+        <is>
+          <t>Balkh</t>
+        </is>
+      </c>
+      <c r="AZ22" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA22" t="n">
+        <v>2</v>
+      </c>
+      <c r="BB22" t="inlineStr">
+        <is>
+          <t>AF2101</t>
+        </is>
+      </c>
       <c r="BC22" t="inlineStr"/>
-      <c r="BD22" t="inlineStr"/>
-      <c r="BE22" t="inlineStr"/>
-      <c r="BF22" t="inlineStr"/>
-      <c r="BG22" t="inlineStr"/>
-      <c r="BH22" t="inlineStr"/>
-      <c r="BI22" t="inlineStr"/>
-      <c r="BJ22" t="inlineStr"/>
-      <c r="BK22" t="inlineStr"/>
-      <c r="BL22" t="n">
+      <c r="BD22" t="inlineStr">
+        <is>
+          <t>Protests ---- Violence against civilians</t>
+        </is>
+      </c>
+      <c r="BE22" t="inlineStr">
+        <is>
+          <t>Peaceful protest ---- Attack</t>
+        </is>
+      </c>
+      <c r="BF22" t="inlineStr">
+        <is>
+          <t>Protesters (Afghanistan) ---- Military Forces of Afghanistan (2021-)</t>
+        </is>
+      </c>
+      <c r="BG22" t="inlineStr">
+        <is>
+          <t>Women (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BH22" t="inlineStr">
+        <is>
+          <t>Civilians (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BI22" t="inlineStr">
+        <is>
+          <t>Students (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BJ22" t="inlineStr">
+        <is>
+          <t>On 17 February 2024, a group of women held a protest in Balkh [coded to Mazar-e-Sharif], against the restrictions imposed by the Taliban on women. They called on participants of the Doha meeting to exert pressure on the Taliban to lift limitations on women's education and employment. ---- On 23 September 2024, a student from Badakhshan province, who was planning to travel to Iran for studies, was beaten and detained by Taliban guards outside the Iranian consulate in Mazar-e-Sharif city, Balkh, following a verbal dispute. The student had been attempting to visit the consulate for over ten days, but the Taliban guards repeatedly denied him entry, leading to the argument. His whereabouts remained unknown.</t>
+        </is>
+      </c>
+      <c r="BK22" t="inlineStr">
+        <is>
+          <t>2024-02-17 ---- 2024-09-23</t>
+        </is>
+      </c>
+      <c r="BL22" t="inlineStr"/>
+      <c r="BM22" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3197,20 +4569,61 @@
       <c r="AV23" t="inlineStr"/>
       <c r="AW23" t="inlineStr"/>
       <c r="AX23" t="inlineStr"/>
-      <c r="AY23" t="inlineStr"/>
-      <c r="AZ23" t="inlineStr"/>
-      <c r="BA23" t="inlineStr"/>
-      <c r="BB23" t="inlineStr"/>
+      <c r="AY23" t="inlineStr">
+        <is>
+          <t>Sar-e Pol</t>
+        </is>
+      </c>
+      <c r="AZ23" t="n">
+        <v>2</v>
+      </c>
+      <c r="BA23" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB23" t="inlineStr">
+        <is>
+          <t>AF2204</t>
+        </is>
+      </c>
       <c r="BC23" t="inlineStr"/>
-      <c r="BD23" t="inlineStr"/>
-      <c r="BE23" t="inlineStr"/>
-      <c r="BF23" t="inlineStr"/>
+      <c r="BD23" t="inlineStr">
+        <is>
+          <t>Violence against civilians</t>
+        </is>
+      </c>
+      <c r="BE23" t="inlineStr">
+        <is>
+          <t>Attack</t>
+        </is>
+      </c>
+      <c r="BF23" t="inlineStr">
+        <is>
+          <t>Unidentified Armed Group (Afghanistan)</t>
+        </is>
+      </c>
       <c r="BG23" t="inlineStr"/>
-      <c r="BH23" t="inlineStr"/>
-      <c r="BI23" t="inlineStr"/>
-      <c r="BJ23" t="inlineStr"/>
-      <c r="BK23" t="inlineStr"/>
-      <c r="BL23" t="n">
+      <c r="BH23" t="inlineStr">
+        <is>
+          <t>Civilians (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BI23" t="inlineStr">
+        <is>
+          <t>Military Forces of Afghanistan (2021-); Students (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BJ23" t="inlineStr">
+        <is>
+          <t>On 3 August 2025, the dead bodies of a Taliban soldier (assumed unarmed) and a religious school student, killed by unidentified persons, were discovered on the highway leading to Sozma Qala district (recently renamed Al-Jihad district), Sar-e-Pol. Motive unknown. Sources said the two were shot dead before their bodies were burned.</t>
+        </is>
+      </c>
+      <c r="BK23" t="inlineStr">
+        <is>
+          <t>2025-08-03</t>
+        </is>
+      </c>
+      <c r="BL23" t="inlineStr"/>
+      <c r="BM23" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3309,20 +4722,61 @@
       <c r="AV24" t="inlineStr"/>
       <c r="AW24" t="inlineStr"/>
       <c r="AX24" t="inlineStr"/>
-      <c r="AY24" t="inlineStr"/>
-      <c r="AZ24" t="inlineStr"/>
-      <c r="BA24" t="inlineStr"/>
-      <c r="BB24" t="inlineStr"/>
+      <c r="AY24" t="inlineStr">
+        <is>
+          <t>Ghor</t>
+        </is>
+      </c>
+      <c r="AZ24" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA24" t="n">
+        <v>4</v>
+      </c>
+      <c r="BB24" t="inlineStr">
+        <is>
+          <t>AF2301</t>
+        </is>
+      </c>
       <c r="BC24" t="inlineStr"/>
-      <c r="BD24" t="inlineStr"/>
-      <c r="BE24" t="inlineStr"/>
-      <c r="BF24" t="inlineStr"/>
+      <c r="BD24" t="inlineStr">
+        <is>
+          <t>Strategic developments ---- Violence against civilians ---- Violence against civilians ---- Strategic developments</t>
+        </is>
+      </c>
+      <c r="BE24" t="inlineStr">
+        <is>
+          <t>Arrests ---- Attack ---- Attack ---- Other</t>
+        </is>
+      </c>
+      <c r="BF24" t="inlineStr">
+        <is>
+          <t>Military Forces of Afghanistan (2021-) ---- Police Forces of Afghanistan (2021-) Vice and Virtue Department ---- Police Forces of Afghanistan (2021-) General Directorate of Intelligence ---- Police Forces of Afghanistan (2021-) General Directorate of Intelligence</t>
+        </is>
+      </c>
       <c r="BG24" t="inlineStr"/>
-      <c r="BH24" t="inlineStr"/>
-      <c r="BI24" t="inlineStr"/>
-      <c r="BJ24" t="inlineStr"/>
-      <c r="BK24" t="inlineStr"/>
-      <c r="BL24" t="n">
+      <c r="BH24" t="inlineStr">
+        <is>
+          <t>Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BI24" t="inlineStr">
+        <is>
+          <t>Journalists (Afghanistan) ---- Students (Afghanistan) ---- Prisoners (Afghanistan) ---- Students (Afghanistan); Teachers (Afghanistan); Women (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BJ24" t="inlineStr">
+        <is>
+          <t>On 4 January 2024, Taliban forces arrested the chief of Saday-e-Adalat Radio in Chighcheran city, Ghor, for broadcasting the UNAMA Mission's message on gender equality in education. The message, shared on social media page of the radio, was deleted post-arrest. The chief was released after one day but refused to comment on the incident to the media. ---- On 3 April 2024, a young student was beaten and seriously wounded by the Taliban's Vice and Virtue Department forces in Gudamha area of Chighcheran (Firuzkoh) city, Ghor, for shaving his beard. He was transferred to the hospital for treatment. ---- Around 26 August 2024, a young man was killed by Taliban intelligence forces in Chighcheran (Firozkoh) city, Ghor. He had been arrested after returning from Iran and was severely tortured for three days. The Taliban claimed he was affiliated with IS, but his family denied the accusation, stating that he was an accounting student in Iran and was busy with his studies. ---- Other: On 25 January 2025, Taliban intelligence forces shut down an English language training center in Lal Wa Sar Jangal district (coded to Lal), Ghor, and arrested its director and four teachers, including a female teacher, due to the center educating girls above the sixth grade. Taliban has banned female education beyond that level (coded separately).</t>
+        </is>
+      </c>
+      <c r="BK24" t="inlineStr">
+        <is>
+          <t>2024-01-04 ---- 2024-04-03 ---- 2024-08-26 ---- 2025-01-25</t>
+        </is>
+      </c>
+      <c r="BL24" t="inlineStr"/>
+      <c r="BM24" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3394,47 +4848,154 @@
       <c r="W25" t="n">
         <v>39.74</v>
       </c>
-      <c r="X25" t="inlineStr"/>
-      <c r="Y25" t="inlineStr"/>
-      <c r="Z25" t="inlineStr"/>
-      <c r="AA25" t="inlineStr"/>
-      <c r="AB25" t="inlineStr"/>
-      <c r="AC25" t="inlineStr"/>
-      <c r="AD25" t="inlineStr"/>
-      <c r="AE25" t="inlineStr"/>
-      <c r="AF25" t="inlineStr"/>
-      <c r="AG25" t="inlineStr"/>
-      <c r="AH25" t="inlineStr"/>
-      <c r="AI25" t="inlineStr"/>
-      <c r="AJ25" t="inlineStr"/>
-      <c r="AK25" t="inlineStr"/>
-      <c r="AL25" t="inlineStr"/>
-      <c r="AM25" t="inlineStr"/>
-      <c r="AN25" t="inlineStr"/>
-      <c r="AO25" t="inlineStr"/>
-      <c r="AP25" t="inlineStr"/>
-      <c r="AQ25" t="inlineStr"/>
-      <c r="AR25" t="inlineStr"/>
-      <c r="AS25" t="inlineStr"/>
-      <c r="AT25" t="inlineStr"/>
-      <c r="AU25" t="inlineStr"/>
-      <c r="AV25" t="inlineStr"/>
+      <c r="X25" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y25" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG25" t="n">
+        <v>25</v>
+      </c>
+      <c r="AH25" t="n">
+        <v>50</v>
+      </c>
+      <c r="AI25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ25" t="n">
+        <v>50</v>
+      </c>
+      <c r="AK25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN25" t="n">
+        <v>6</v>
+      </c>
+      <c r="AO25" t="inlineStr">
+        <is>
+          <t>2025-05-19 ---- 2025-05-19 ---- 2025-05-07 ---- 2025-05-07 ---- 2025-02-26 ---- 2025-01-13</t>
+        </is>
+      </c>
+      <c r="AP25" t="inlineStr">
+        <is>
+          <t>May 2025: Five educators and a head of programme were arrested and sentenced to prison by Taliban authorities for ‚Äúteaching Christian content‚Äù. ---- As reported May 2025: An education centre was closed and its staff arrested by the Taliban. ---- May 2025: Around 25 students were poisoned at a school allegedly by the Taliban to deter girls from going to school. ---- May 2025: Around 25 students were poisoned at a school allegedly by the Taliban to deter girls from going to school. ---- 26 February 2025: Nine teachers were summoned to court by Taliban authorities then subsequently detained. They were accused of promoting a foreign culture and that their curriculum lacked sufficient religious content. ---- January 2025: Nine teachers were arrested by Taliban authorities and released three days later. They were accused of promoting a foreign culture and that their curriculum lacked sufficient religious content.</t>
+        </is>
+      </c>
+      <c r="AQ25" t="inlineStr">
+        <is>
+          <t>Unspecified Location ---- Education Building  ---- Education Building  ---- Education Building  ---- Other ---- Unspecified Location</t>
+        </is>
+      </c>
+      <c r="AR25" t="inlineStr">
+        <is>
+          <t>Other ---- Other ---- Police ---- Police ---- Police ---- Other</t>
+        </is>
+      </c>
+      <c r="AS25" t="inlineStr">
+        <is>
+          <t>Islamic Emirate of Afghanistan ---- Islamic Emirate of Afghanistan ---- Islamic Emirate of Afghanistan ---- Islamic Emirate of Afghanistan ---- Islamic Emirate of Afghanistan ---- Islamic Emirate of Afghanistan</t>
+        </is>
+      </c>
+      <c r="AT25" t="inlineStr">
+        <is>
+          <t>Firearms ---- Firearms ---- Other Weapon ---- Other Weapon ---- Firearms ---- Firearms</t>
+        </is>
+      </c>
+      <c r="AU25" t="inlineStr">
+        <is>
+          <t>Not Applicable ---- School: No Further Details ---- Secondary School ---- Primary School ---- Not Applicable ---- Not Applicable</t>
+        </is>
+      </c>
+      <c r="AV25" t="inlineStr">
+        <is>
+          <t>NoInformation ---- NoInformation ---- NoInformation ---- Freed</t>
+        </is>
+      </c>
       <c r="AW25" t="inlineStr"/>
       <c r="AX25" t="inlineStr"/>
-      <c r="AY25" t="inlineStr"/>
-      <c r="AZ25" t="inlineStr"/>
-      <c r="BA25" t="inlineStr"/>
-      <c r="BB25" t="inlineStr"/>
+      <c r="AY25" t="inlineStr">
+        <is>
+          <t>Daykundi</t>
+        </is>
+      </c>
+      <c r="AZ25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA25" t="n">
+        <v>4</v>
+      </c>
+      <c r="BB25" t="inlineStr">
+        <is>
+          <t>AF2405</t>
+        </is>
+      </c>
       <c r="BC25" t="inlineStr"/>
-      <c r="BD25" t="inlineStr"/>
-      <c r="BE25" t="inlineStr"/>
-      <c r="BF25" t="inlineStr"/>
+      <c r="BD25" t="inlineStr">
+        <is>
+          <t>Violence against civilians ---- Protests ---- Violence against civilians ---- Violence against civilians</t>
+        </is>
+      </c>
+      <c r="BE25" t="inlineStr">
+        <is>
+          <t>Attack ---- Peaceful protest ---- Attack ---- Abduction/forced disappearance</t>
+        </is>
+      </c>
+      <c r="BF25" t="inlineStr">
+        <is>
+          <t>Unidentified Armed Group (Afghanistan) ---- Protesters (Afghanistan) ---- Unidentified Armed Group (Afghanistan) ---- Military Forces of Afghanistan (2021-)</t>
+        </is>
+      </c>
       <c r="BG25" t="inlineStr"/>
-      <c r="BH25" t="inlineStr"/>
-      <c r="BI25" t="inlineStr"/>
-      <c r="BJ25" t="inlineStr"/>
-      <c r="BK25" t="inlineStr"/>
-      <c r="BL25" t="n">
+      <c r="BH25" t="inlineStr">
+        <is>
+          <t>Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BI25" t="inlineStr">
+        <is>
+          <t>Students (Afghanistan); Teachers (Afghanistan); Women (Afghanistan) ---- Women (Afghanistan); Students (Afghanistan) ---- Teachers (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BJ25" t="inlineStr">
+        <is>
+          <t>On 16 May 2024, at least 80-90 female students and 1-15 female teachers were poisoned at a high school in the Taymuran area of Kiti district, Daykundi. They were moved to the district and provincial hospitals for treatment, with at least three students in critical condition. A teacher said they smelled 'a bad smell' before they felt ill. The cause is unknown. ---- Around 30 July 2024 (as reported), local residents from several villages of Daikundi [coded to Nili] province protested against the proposed location for a new school building, arguing its remote location and significant travel challenges for children. Taliban's education chief insisted on the school building at the selected site. ---- On 7 May 2025, at least 50 female students were poisoned at a high school in Kiti district, Daykundi. The students were transferred to local clinics and health centers. One student's father said she fell ill after inhaling a strong odor resembling acid. Locals claimed the incident was a part of a Taliban tactic to intimidate girls and deter them from attending school by instilling fear among students and their families. Female students were also poisoned in the same district last year (coded separately). ---- Around 19 May 2025 (as reported), Taliban forces arrested several teachers from the Ufoq Naw English language training center in Sang-e-Takht district, Daykundi, and shut down the center. The whereabouts of the detained teachers remained unknown.</t>
+        </is>
+      </c>
+      <c r="BK25" t="inlineStr">
+        <is>
+          <t>2024-05-16 ---- 2024-07-30 ---- 2025-05-07 ---- 2025-05-19</t>
+        </is>
+      </c>
+      <c r="BL25" t="inlineStr"/>
+      <c r="BM25" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3546,7 +5107,8 @@
       <c r="BI26" t="inlineStr"/>
       <c r="BJ26" t="inlineStr"/>
       <c r="BK26" t="inlineStr"/>
-      <c r="BL26" t="n">
+      <c r="BL26" t="inlineStr"/>
+      <c r="BM26" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3658,7 +5220,8 @@
       <c r="BI27" t="inlineStr"/>
       <c r="BJ27" t="inlineStr"/>
       <c r="BK27" t="inlineStr"/>
-      <c r="BL27" t="n">
+      <c r="BL27" t="inlineStr"/>
+      <c r="BM27" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3757,20 +5320,61 @@
       <c r="AV28" t="inlineStr"/>
       <c r="AW28" t="inlineStr"/>
       <c r="AX28" t="inlineStr"/>
-      <c r="AY28" t="inlineStr"/>
-      <c r="AZ28" t="inlineStr"/>
-      <c r="BA28" t="inlineStr"/>
-      <c r="BB28" t="inlineStr"/>
+      <c r="AY28" t="inlineStr">
+        <is>
+          <t>Kandahar</t>
+        </is>
+      </c>
+      <c r="AZ28" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA28" t="n">
+        <v>2</v>
+      </c>
+      <c r="BB28" t="inlineStr">
+        <is>
+          <t>AF2701</t>
+        </is>
+      </c>
       <c r="BC28" t="inlineStr"/>
-      <c r="BD28" t="inlineStr"/>
-      <c r="BE28" t="inlineStr"/>
-      <c r="BF28" t="inlineStr"/>
+      <c r="BD28" t="inlineStr">
+        <is>
+          <t>Strategic developments ---- Violence against civilians</t>
+        </is>
+      </c>
+      <c r="BE28" t="inlineStr">
+        <is>
+          <t>Other ---- Attack</t>
+        </is>
+      </c>
+      <c r="BF28" t="inlineStr">
+        <is>
+          <t>Government of Afghanistan (2021-) ---- Unidentified Armed Group (Afghanistan)</t>
+        </is>
+      </c>
       <c r="BG28" t="inlineStr"/>
-      <c r="BH28" t="inlineStr"/>
-      <c r="BI28" t="inlineStr"/>
-      <c r="BJ28" t="inlineStr"/>
-      <c r="BK28" t="inlineStr"/>
-      <c r="BL28" t="n">
+      <c r="BH28" t="inlineStr">
+        <is>
+          <t>Civilians (Afghanistan) ---- Civilians (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BI28" t="inlineStr">
+        <is>
+          <t>Students (Afghanistan); Women (Afghanistan) ---- Government of Afghanistan (2021-)</t>
+        </is>
+      </c>
+      <c r="BJ28" t="inlineStr">
+        <is>
+          <t>Other: Around 22 February 2024 (as reported), Taliban issued an unofficial directive and ordered school principals in Kandahar province to prohibit female students above the age of 10 from attending school. Previous nationwide directives banned girls to attend schools above the sixth grade, as the Taliban had mandated that students in grades four to six wear face coverings during their commute to school. ---- On 2 June 2025, unknown gunment shot dead the Taliban's head of education for Dand district in the Yakh Karez area of PD15 in Kandahar city, while riding a motorcycle from his home to the mosque. Motive unknown. No group has claimed responsibility. While the Taliban stated that the attackers were armed robbers, local sources reported that no belongings were taken from the victim during the incident</t>
+        </is>
+      </c>
+      <c r="BK28" t="inlineStr">
+        <is>
+          <t>2024-02-22 ---- 2025-06-02</t>
+        </is>
+      </c>
+      <c r="BL28" t="inlineStr"/>
+      <c r="BM28" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3882,7 +5486,8 @@
       <c r="BI29" t="inlineStr"/>
       <c r="BJ29" t="inlineStr"/>
       <c r="BK29" t="inlineStr"/>
-      <c r="BL29" t="n">
+      <c r="BL29" t="inlineStr"/>
+      <c r="BM29" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3981,20 +5586,57 @@
       <c r="AV30" t="inlineStr"/>
       <c r="AW30" t="inlineStr"/>
       <c r="AX30" t="inlineStr"/>
-      <c r="AY30" t="inlineStr"/>
-      <c r="AZ30" t="inlineStr"/>
-      <c r="BA30" t="inlineStr"/>
-      <c r="BB30" t="inlineStr"/>
+      <c r="AY30" t="inlineStr">
+        <is>
+          <t>Faryab</t>
+        </is>
+      </c>
+      <c r="AZ30" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA30" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB30" t="inlineStr">
+        <is>
+          <t>AF2901</t>
+        </is>
+      </c>
       <c r="BC30" t="inlineStr"/>
-      <c r="BD30" t="inlineStr"/>
-      <c r="BE30" t="inlineStr"/>
-      <c r="BF30" t="inlineStr"/>
+      <c r="BD30" t="inlineStr">
+        <is>
+          <t>Violence against civilians</t>
+        </is>
+      </c>
+      <c r="BE30" t="inlineStr">
+        <is>
+          <t>Attack</t>
+        </is>
+      </c>
+      <c r="BF30" t="inlineStr">
+        <is>
+          <t>Military Forces of Afghanistan (2021-)</t>
+        </is>
+      </c>
       <c r="BG30" t="inlineStr"/>
-      <c r="BH30" t="inlineStr"/>
+      <c r="BH30" t="inlineStr">
+        <is>
+          <t>Civilians (Afghanistan)</t>
+        </is>
+      </c>
       <c r="BI30" t="inlineStr"/>
-      <c r="BJ30" t="inlineStr"/>
-      <c r="BK30" t="inlineStr"/>
-      <c r="BL30" t="n">
+      <c r="BJ30" t="inlineStr">
+        <is>
+          <t>On 27 August 2024, a Taliban criminal command member shot and killed a young man near Abu Abid Jozjani School in Maimana city, Faryab. Motive unknown. The Taliban arrested the accused member.</t>
+        </is>
+      </c>
+      <c r="BK30" t="inlineStr">
+        <is>
+          <t>2024-08-27</t>
+        </is>
+      </c>
+      <c r="BL30" t="inlineStr"/>
+      <c r="BM30" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4093,20 +5735,61 @@
       <c r="AV31" t="inlineStr"/>
       <c r="AW31" t="inlineStr"/>
       <c r="AX31" t="inlineStr"/>
-      <c r="AY31" t="inlineStr"/>
-      <c r="AZ31" t="inlineStr"/>
-      <c r="BA31" t="inlineStr"/>
-      <c r="BB31" t="inlineStr"/>
+      <c r="AY31" t="inlineStr">
+        <is>
+          <t>Helmand</t>
+        </is>
+      </c>
+      <c r="AZ31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA31" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB31" t="inlineStr">
+        <is>
+          <t>AF3001</t>
+        </is>
+      </c>
       <c r="BC31" t="inlineStr"/>
-      <c r="BD31" t="inlineStr"/>
-      <c r="BE31" t="inlineStr"/>
-      <c r="BF31" t="inlineStr"/>
+      <c r="BD31" t="inlineStr">
+        <is>
+          <t>Strategic developments</t>
+        </is>
+      </c>
+      <c r="BE31" t="inlineStr">
+        <is>
+          <t>Arrests</t>
+        </is>
+      </c>
+      <c r="BF31" t="inlineStr">
+        <is>
+          <t>Police Forces of Afghanistan (2021-) General Directorate of Intelligence</t>
+        </is>
+      </c>
       <c r="BG31" t="inlineStr"/>
-      <c r="BH31" t="inlineStr"/>
-      <c r="BI31" t="inlineStr"/>
-      <c r="BJ31" t="inlineStr"/>
-      <c r="BK31" t="inlineStr"/>
-      <c r="BL31" t="n">
+      <c r="BH31" t="inlineStr">
+        <is>
+          <t>Civilians (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BI31" t="inlineStr">
+        <is>
+          <t>Muslim Group (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BJ31" t="inlineStr">
+        <is>
+          <t>On 3 May 2025, Taliban intelligence forces arrested a prominent religious scholar in Lashkargah city, Helmand, upon his arrival in Afghanistan from Egypt. Taliban sentenced him to eight months in prison, along with a two year ban on foreign travel. He had previously been arrested as well. The scholar is a graduate of Al-Azhar University in Cairo and a well-known cleric and influential figure in the province. He had founded a religious seminary in Helmand and also opened cafes and restaurants in Helmand and Kandahar, aiming to create community spaces for youth. While the exact motive for his arrest remained unclear, he is known for his criticism of Taliban policies particularly the ban on girls' education and had recently discussed about bay'ah (allegiance) and leadership in an interview. He was released on 3 June 2025, but it is unknown whether the travel ban is still in effect.</t>
+        </is>
+      </c>
+      <c r="BK31" t="inlineStr">
+        <is>
+          <t>2025-05-03</t>
+        </is>
+      </c>
+      <c r="BL31" t="inlineStr"/>
+      <c r="BM31" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4205,20 +5888,57 @@
       <c r="AV32" t="inlineStr"/>
       <c r="AW32" t="inlineStr"/>
       <c r="AX32" t="inlineStr"/>
-      <c r="AY32" t="inlineStr"/>
-      <c r="AZ32" t="inlineStr"/>
-      <c r="BA32" t="inlineStr"/>
-      <c r="BB32" t="inlineStr"/>
+      <c r="AY32" t="inlineStr">
+        <is>
+          <t>Badghis</t>
+        </is>
+      </c>
+      <c r="AZ32" t="n">
+        <v>3</v>
+      </c>
+      <c r="BA32" t="n">
+        <v>2</v>
+      </c>
+      <c r="BB32" t="inlineStr">
+        <is>
+          <t>AF3101</t>
+        </is>
+      </c>
       <c r="BC32" t="inlineStr"/>
-      <c r="BD32" t="inlineStr"/>
-      <c r="BE32" t="inlineStr"/>
-      <c r="BF32" t="inlineStr"/>
+      <c r="BD32" t="inlineStr">
+        <is>
+          <t>Battles ---- Explosions/Remote violence</t>
+        </is>
+      </c>
+      <c r="BE32" t="inlineStr">
+        <is>
+          <t>Armed clash ---- Grenade</t>
+        </is>
+      </c>
+      <c r="BF32" t="inlineStr">
+        <is>
+          <t>Unidentified Armed Group (Afghanistan) ---- National Resistance Front</t>
+        </is>
+      </c>
       <c r="BG32" t="inlineStr"/>
-      <c r="BH32" t="inlineStr"/>
+      <c r="BH32" t="inlineStr">
+        <is>
+          <t>Military Forces of Afghanistan (2021-) ---- Military Forces of Afghanistan (2021-)</t>
+        </is>
+      </c>
       <c r="BI32" t="inlineStr"/>
-      <c r="BJ32" t="inlineStr"/>
-      <c r="BK32" t="inlineStr"/>
-      <c r="BL32" t="n">
+      <c r="BJ32" t="inlineStr">
+        <is>
+          <t>On 28 July 2024, unidentified armed men shot dead a Taliban member responsible for the education and training of the Taliban security command in Sarpol area of Tagab Alam district [unfound, coded to provincial capital Qala-i-Now], Badghis. The motive remained unclear. Taliban arrested one person in connection with the incident. ---- On 19 September 2024, two Taliban members were killed and three others were wounded following a hand grenade attack by the NRF targeting the Taliban's Al-Farooq Corps Brigade in Badghis (coded to Qala-i-Now) province. Local sources confirmed the attack. The Taliban arrested their head of education for Ab Kamari district of Badghis, in connection with the incident.</t>
+        </is>
+      </c>
+      <c r="BK32" t="inlineStr">
+        <is>
+          <t>2024-07-28 ---- 2024-09-19</t>
+        </is>
+      </c>
+      <c r="BL32" t="inlineStr"/>
+      <c r="BM32" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4290,47 +6010,154 @@
       <c r="W33" t="n">
         <v>39.89</v>
       </c>
-      <c r="X33" t="inlineStr"/>
-      <c r="Y33" t="inlineStr"/>
-      <c r="Z33" t="inlineStr"/>
-      <c r="AA33" t="inlineStr"/>
-      <c r="AB33" t="inlineStr"/>
-      <c r="AC33" t="inlineStr"/>
-      <c r="AD33" t="inlineStr"/>
-      <c r="AE33" t="inlineStr"/>
-      <c r="AF33" t="inlineStr"/>
-      <c r="AG33" t="inlineStr"/>
-      <c r="AH33" t="inlineStr"/>
-      <c r="AI33" t="inlineStr"/>
-      <c r="AJ33" t="inlineStr"/>
-      <c r="AK33" t="inlineStr"/>
-      <c r="AL33" t="inlineStr"/>
-      <c r="AM33" t="inlineStr"/>
-      <c r="AN33" t="inlineStr"/>
-      <c r="AO33" t="inlineStr"/>
-      <c r="AP33" t="inlineStr"/>
-      <c r="AQ33" t="inlineStr"/>
-      <c r="AR33" t="inlineStr"/>
-      <c r="AS33" t="inlineStr"/>
-      <c r="AT33" t="inlineStr"/>
-      <c r="AU33" t="inlineStr"/>
+      <c r="X33" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH33" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO33" t="inlineStr">
+        <is>
+          <t>2024-02-21</t>
+        </is>
+      </c>
+      <c r="AP33" t="inlineStr">
+        <is>
+          <t>February 2024: the director of a school was attacked and shot dead when unidentified assailants attacked the school. Two armed men reportedly assaulted some staff members.</t>
+        </is>
+      </c>
+      <c r="AQ33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Education Building </t>
+        </is>
+      </c>
+      <c r="AR33" t="inlineStr">
+        <is>
+          <t>Criminal</t>
+        </is>
+      </c>
+      <c r="AS33" t="inlineStr">
+        <is>
+          <t>Unidentified Armed Actor</t>
+        </is>
+      </c>
+      <c r="AT33" t="inlineStr">
+        <is>
+          <t>Fist and Foot</t>
+        </is>
+      </c>
+      <c r="AU33" t="inlineStr">
+        <is>
+          <t>School: No Further Details</t>
+        </is>
+      </c>
       <c r="AV33" t="inlineStr"/>
       <c r="AW33" t="inlineStr"/>
       <c r="AX33" t="inlineStr"/>
-      <c r="AY33" t="inlineStr"/>
-      <c r="AZ33" t="inlineStr"/>
-      <c r="BA33" t="inlineStr"/>
-      <c r="BB33" t="inlineStr"/>
+      <c r="AY33" t="inlineStr">
+        <is>
+          <t>Herat</t>
+        </is>
+      </c>
+      <c r="AZ33" t="n">
+        <v>5</v>
+      </c>
+      <c r="BA33" t="n">
+        <v>7</v>
+      </c>
+      <c r="BB33" t="inlineStr">
+        <is>
+          <t>AF3201</t>
+        </is>
+      </c>
       <c r="BC33" t="inlineStr"/>
-      <c r="BD33" t="inlineStr"/>
-      <c r="BE33" t="inlineStr"/>
-      <c r="BF33" t="inlineStr"/>
-      <c r="BG33" t="inlineStr"/>
-      <c r="BH33" t="inlineStr"/>
-      <c r="BI33" t="inlineStr"/>
-      <c r="BJ33" t="inlineStr"/>
-      <c r="BK33" t="inlineStr"/>
-      <c r="BL33" t="n">
+      <c r="BD33" t="inlineStr">
+        <is>
+          <t>Violence against civilians ---- Violence against civilians ---- Strategic developments ---- Battles ---- Violence against civilians ---- Protests ---- Strategic developments</t>
+        </is>
+      </c>
+      <c r="BE33" t="inlineStr">
+        <is>
+          <t>Attack ---- Attack ---- Arrests ---- Armed clash ---- Attack ---- Protest with intervention ---- Other</t>
+        </is>
+      </c>
+      <c r="BF33" t="inlineStr">
+        <is>
+          <t>Unidentified Armed Group (Afghanistan) ---- Unidentified Armed Group (Afghanistan) ---- Police Forces of Afghanistan (2021-) Vice and Virtue Department ---- National Resistance Front ---- Military Forces of Afghanistan (2021-) ---- Protesters (Afghanistan) ---- Government of Afghanistan (2021-)</t>
+        </is>
+      </c>
+      <c r="BG33" t="inlineStr">
+        <is>
+          <t>Health Workers (Afghanistan); Students (Afghanistan); Women (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BH33" t="inlineStr">
+        <is>
+          <t>Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Civilians (Afghanistan) ---- Military Forces of Afghanistan (2021-) ---- Civilians (Afghanistan) ---- Military Forces of Afghanistan (2021-) ---- Civilians (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BI33" t="inlineStr">
+        <is>
+          <t>Muslim Group (Afghanistan); Teachers (Afghanistan) ---- Teachers (Afghanistan); Labor Group (Afghanistan) ---- Teachers (Afghanistan) ---- Prisoners (Afghanistan); Teachers (Afghanistan) ---- Students (Afghanistan); Women (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BJ33" t="inlineStr">
+        <is>
+          <t>On 25 January 2024, a religious scholar was shot and killed by unknown armed men in Herat city. Attackers managed to escape. Motive unknown. ---- On 21 February 2024, unknown armed men attacked at the 'Roshan Zamiran' private school, shot dead the principal and beat several other employees of the school in Qoul Ordu area of Herat city. An eyewitness said that the attackers, although took a number of the employees' cell phones, they did not appear to be robbers. He claimed that it was a targeted attack. Event took place in the presence of teachers, no further information. ---- On 8 May 2024, Members of the Taliban's Vice and Virtue department arrested and imprisoned six university professors from the agricultural institute in Herat city, subjecting them to humiliation and insults. They were accused of shaving or having short beards after the Taliban entered the classrooms and measured the teachers' beards. ---- On 19 August 2024, two Taliban Al-Farooq Corps members were killed following an attack by National Resistance Front militants on a Taliban position in Sultan Bayazid Bastami Mosque Street near Ustad Heneriar High School in the Nowabad area of Herat city. No casualties from NRF. ---- On 27 November 2024, Taliban arrested a teacher/engineer in the Bagh Murad area of Herat city. His body was handed to his family a day later with signs of torture. Motive unknown. ---- On 5 December 2024, a number of female students held a protest in Herat city to denounce Taliban's decision to close all public and private medical institutes for female medical education (coded separately). Taliban confiscated the protest banners. ---- Other: On 23 December 2024, the Taliban, following an order from their leader Mullah Hibatullah Akhundzada, banned girls above sixth grade from attending private educational centers in Herat province. These centers were providing lessons in English and other school subjects. This follows previous nationwide decrees prohibiting girls from attending schools above the sixth grade, as well as barring them from universities and health institutes.</t>
+        </is>
+      </c>
+      <c r="BK33" t="inlineStr">
+        <is>
+          <t>2024-01-25 ---- 2024-02-21 ---- 2024-05-08 ---- 2024-08-19 ---- 2024-11-27 ---- 2024-12-05 ---- 2024-12-23</t>
+        </is>
+      </c>
+      <c r="BL33" t="inlineStr"/>
+      <c r="BM33" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4429,20 +6256,61 @@
       <c r="AV34" t="inlineStr"/>
       <c r="AW34" t="inlineStr"/>
       <c r="AX34" t="inlineStr"/>
-      <c r="AY34" t="inlineStr"/>
-      <c r="AZ34" t="inlineStr"/>
-      <c r="BA34" t="inlineStr"/>
-      <c r="BB34" t="inlineStr"/>
+      <c r="AY34" t="inlineStr">
+        <is>
+          <t>Farah</t>
+        </is>
+      </c>
+      <c r="AZ34" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA34" t="n">
+        <v>2</v>
+      </c>
+      <c r="BB34" t="inlineStr">
+        <is>
+          <t>AF3302</t>
+        </is>
+      </c>
       <c r="BC34" t="inlineStr"/>
-      <c r="BD34" t="inlineStr"/>
-      <c r="BE34" t="inlineStr"/>
-      <c r="BF34" t="inlineStr"/>
+      <c r="BD34" t="inlineStr">
+        <is>
+          <t>Strategic developments ---- Battles</t>
+        </is>
+      </c>
+      <c r="BE34" t="inlineStr">
+        <is>
+          <t>Other ---- Armed clash</t>
+        </is>
+      </c>
+      <c r="BF34" t="inlineStr">
+        <is>
+          <t>Unidentified Armed Group (Afghanistan) ---- National Resistance Front</t>
+        </is>
+      </c>
       <c r="BG34" t="inlineStr"/>
-      <c r="BH34" t="inlineStr"/>
-      <c r="BI34" t="inlineStr"/>
-      <c r="BJ34" t="inlineStr"/>
-      <c r="BK34" t="inlineStr"/>
-      <c r="BL34" t="n">
+      <c r="BH34" t="inlineStr">
+        <is>
+          <t>Civilians (Afghanistan) ---- Military Forces of Afghanistan (2021-)</t>
+        </is>
+      </c>
+      <c r="BI34" t="inlineStr">
+        <is>
+          <t>Students (Afghanistan)</t>
+        </is>
+      </c>
+      <c r="BJ34" t="inlineStr">
+        <is>
+          <t>Explosive remnants of war: On 1 April 2024, three children, students, were wounded when a mortar shell, remnants of war, exploded in the Ganjgin area of Pushtrud district, Farah. The children were playing with it when it exploded. ---- On 17 August 2024, one Taliban drug management member was killed and two others were wounded following an attack by National Resistance Front militants at their checkpoint in Engineer Hatem's Street behind Abu Zar Al-Ghafari Mosque within the PD1 of Farah city. In another attack, two Taliban members were wounded, a weapon was seized, and a Taliban vehicle was also destroyed following an attack in front of the Jamia Al-Huda School on the Social Affairs Directorate Road in PD4 of Farah City. No casualties from NRF.</t>
+        </is>
+      </c>
+      <c r="BK34" t="inlineStr">
+        <is>
+          <t>2024-04-01 ---- 2024-08-17</t>
+        </is>
+      </c>
+      <c r="BL34" t="inlineStr"/>
+      <c r="BM34" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4514,47 +6382,142 @@
       <c r="W35" t="n">
         <v>39.65</v>
       </c>
-      <c r="X35" t="inlineStr"/>
-      <c r="Y35" t="inlineStr"/>
-      <c r="Z35" t="inlineStr"/>
-      <c r="AA35" t="inlineStr"/>
-      <c r="AB35" t="inlineStr"/>
-      <c r="AC35" t="inlineStr"/>
-      <c r="AD35" t="inlineStr"/>
-      <c r="AE35" t="inlineStr"/>
-      <c r="AF35" t="inlineStr"/>
-      <c r="AG35" t="inlineStr"/>
-      <c r="AH35" t="inlineStr"/>
-      <c r="AI35" t="inlineStr"/>
-      <c r="AJ35" t="inlineStr"/>
-      <c r="AK35" t="inlineStr"/>
-      <c r="AL35" t="inlineStr"/>
-      <c r="AM35" t="inlineStr"/>
-      <c r="AN35" t="inlineStr"/>
-      <c r="AO35" t="inlineStr"/>
-      <c r="AP35" t="inlineStr"/>
-      <c r="AQ35" t="inlineStr"/>
-      <c r="AR35" t="inlineStr"/>
-      <c r="AS35" t="inlineStr"/>
-      <c r="AT35" t="inlineStr"/>
-      <c r="AU35" t="inlineStr"/>
+      <c r="X35" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y35" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO35" t="inlineStr">
+        <is>
+          <t>2024-02-18</t>
+        </is>
+      </c>
+      <c r="AP35" t="inlineStr">
+        <is>
+          <t>February 2024: a school bordering Iran was turned into a military base by Taliban forces. A Taliban member confirmed that the military base was built after recent border tensions with Iran.</t>
+        </is>
+      </c>
+      <c r="AQ35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Education Building </t>
+        </is>
+      </c>
+      <c r="AR35" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="AS35" t="inlineStr">
+        <is>
+          <t>Islamic Emirate of Afghanistan</t>
+        </is>
+      </c>
+      <c r="AT35" t="inlineStr">
+        <is>
+          <t>Firearms</t>
+        </is>
+      </c>
+      <c r="AU35" t="inlineStr">
+        <is>
+          <t>School: No Further Details</t>
+        </is>
+      </c>
       <c r="AV35" t="inlineStr"/>
       <c r="AW35" t="inlineStr"/>
       <c r="AX35" t="inlineStr"/>
-      <c r="AY35" t="inlineStr"/>
-      <c r="AZ35" t="inlineStr"/>
-      <c r="BA35" t="inlineStr"/>
-      <c r="BB35" t="inlineStr"/>
+      <c r="AY35" t="inlineStr">
+        <is>
+          <t>Nimruz</t>
+        </is>
+      </c>
+      <c r="AZ35" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA35" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB35" t="inlineStr">
+        <is>
+          <t>AF3401</t>
+        </is>
+      </c>
       <c r="BC35" t="inlineStr"/>
-      <c r="BD35" t="inlineStr"/>
-      <c r="BE35" t="inlineStr"/>
-      <c r="BF35" t="inlineStr"/>
+      <c r="BD35" t="inlineStr">
+        <is>
+          <t>Strategic developments</t>
+        </is>
+      </c>
+      <c r="BE35" t="inlineStr">
+        <is>
+          <t>Headquarters or base established</t>
+        </is>
+      </c>
+      <c r="BF35" t="inlineStr">
+        <is>
+          <t>Military Forces of Afghanistan (2021-)</t>
+        </is>
+      </c>
       <c r="BG35" t="inlineStr"/>
       <c r="BH35" t="inlineStr"/>
       <c r="BI35" t="inlineStr"/>
-      <c r="BJ35" t="inlineStr"/>
-      <c r="BK35" t="inlineStr"/>
-      <c r="BL35" t="n">
+      <c r="BJ35" t="inlineStr">
+        <is>
+          <t>Around 18 February 2024 (as reported), Taliban forces turned a school into a military base in Khwabgah village of Char Burjak district, Nimruz, bordering with Iran. A Taliban member confirmed that the military base was built after the recent border tensions with Iran.</t>
+        </is>
+      </c>
+      <c r="BK35" t="inlineStr">
+        <is>
+          <t>2024-02-18</t>
+        </is>
+      </c>
+      <c r="BL35" t="inlineStr"/>
+      <c r="BM35" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4564,10 +6527,10 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C9824523CAB29F4DA646F20BAFE41B4C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9c972c102b01d47663811fb2ebdbd1e4">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5940141-1bc9-4c17-b1bc-e50f6b2083d6" xmlns:ns3="14cbb838-50ff-4dab-9c3f-cddf75f03c13" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="bd0e8b72e466adcc572d3af37c1ebe05" ns2:_="" ns3:_="">
-    <xsd:import namespace="b5940141-1bc9-4c17-b1bc-e50f6b2083d6"/>
-    <xsd:import namespace="14cbb838-50ff-4dab-9c3f-cddf75f03c13"/>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100DE51FB2AFBB2DD429D3D11FE759FFC43" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1354c8e90e28409d311bbba5db8dc335">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f4877444-78fa-4cfa-bafc-d6c64fafc061" xmlns:ns3="d0fa6634-326e-4532-91a2-52bea7ac9212" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="dbb4473bd7833dc3543803a005841490" ns2:_="" ns3:_="">
+    <xsd:import namespace="f4877444-78fa-4cfa-bafc-d6c64fafc061"/>
+    <xsd:import namespace="d0fa6634-326e-4532-91a2-52bea7ac9212"/>
     <xsd:element name="properties">
       <xsd:complexType>
         <xsd:sequence>
@@ -4579,13 +6542,15 @@
                 <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
                 <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
                 <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
@@ -4594,7 +6559,7 @@
       </xsd:complexType>
     </xsd:element>
   </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b5940141-1bc9-4c17-b1bc-e50f6b2083d6" elementFormDefault="qualified">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="f4877444-78fa-4cfa-bafc-d6c64fafc061" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
@@ -4612,52 +6577,57 @@
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="14" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="4d06f0b5-5743-41f2-90d3-b12c8ffc7f36" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+    <xsd:element name="MediaServiceDateTaken" ma:index="13" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="14" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="15" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="16" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="18" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="4d06f0b5-5743-41f2-90d3-b12c8ffc7f36" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
       <xsd:complexType>
         <xsd:sequence>
           <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
         </xsd:sequence>
       </xsd:complexType>
     </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+    <xsd:element name="MediaServiceOCR" ma:index="20" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note">
           <xsd:maxLength value="255"/>
         </xsd:restriction>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+    <xsd:element name="MediaServiceSearchProperties" ma:index="21" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="22" nillable="true" ma:displayName="Location" ma:description="" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="18" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="19" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="20" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceBillingMetadata" ma:index="21" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="23" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
   </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="14cbb838-50ff-4dab-9c3f-cddf75f03c13" elementFormDefault="qualified">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d0fa6634-326e-4532-91a2-52bea7ac9212" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <xsd:element name="SharedWithUsers" ma:index="11" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
@@ -4685,6 +6655,17 @@
           <xsd:maxLength value="255"/>
         </xsd:restriction>
       </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="TaxCatchAll" ma:index="19" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{d6bd4e25-e667-4943-8e38-5db701f530ee}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="d0fa6634-326e-4532-91a2-52bea7ac9212">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
     </xsd:element>
   </xsd:schema>
   <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
@@ -4798,7 +6779,8 @@
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5940141-1bc9-4c17-b1bc-e50f6b2083d6">
+    <TaxCatchAll xmlns="d0fa6634-326e-4532-91a2-52bea7ac9212" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f4877444-78fa-4cfa-bafc-d6c64fafc061">
       <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
@@ -4806,13 +6788,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0AE1F0C9-8E9C-4891-9430-D9EECB706FD4}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3F2A3E3-57C7-4EFF-9D76-2F26EB9F36FB}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3C69544C-03A5-4BC3-8C5A-F52E2F41EFB7}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5BD55AD2-34E8-4875-92E0-247C3AD93496}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6AAA37A9-C1A6-435C-9331-BB5415846613}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AE095164-DE9F-4D09-93F8-F42A26C0800B}"/>
 </file>
</xml_diff>